<commit_message>
fix: align batch inputs and location eligibility
</commit_message>
<xml_diff>
--- a/data/templates/model_dataset_template.xlsx
+++ b/data/templates/model_dataset_template.xlsx
@@ -1540,7 +1540,7 @@
     <numFmt numFmtId="0" formatCode="General"/>
     <numFmt numFmtId="59" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -1556,39 +1556,16 @@
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="16"/>
-      <color indexed="8"/>
-      <name val="Aptos"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Aptos"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Aptos"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="9"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1598,76 +1575,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="10"/>
+        <color indexed="9"/>
       </left>
       <right style="thin">
-        <color indexed="10"/>
+        <color indexed="9"/>
       </right>
       <top style="thin">
-        <color indexed="10"/>
+        <color indexed="9"/>
       </top>
       <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
+        <color indexed="9"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1677,62 +1594,23 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="59" fontId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -1752,8 +1630,7 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="ffa5a5a5"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1952,7 +1829,7 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="19050" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
@@ -1989,10 +1866,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -2231,7 +2108,7 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="19050" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
@@ -2540,10 +2417,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -2786,7 +2663,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E35"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="27" style="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="1" customWidth="1"/>
@@ -2803,445 +2680,445 @@
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="4"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" t="s" s="6">
+      <c r="A3" t="s" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="4"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" t="s" s="8">
+      <c r="A4" t="s" s="2">
         <v>2</v>
       </c>
-      <c r="B4" t="s" s="9">
+      <c r="B4" t="s" s="2">
         <v>3</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="11"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" t="s" s="8">
+      <c r="A5" t="s" s="2">
         <v>4</v>
       </c>
-      <c r="B5" t="s" s="9">
+      <c r="B5" t="s" s="2">
         <v>5</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="11"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" t="s" s="8">
+      <c r="A6" t="s" s="2">
         <v>6</v>
       </c>
-      <c r="B6" t="s" s="9">
+      <c r="B6" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="11"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" t="s" s="8">
+      <c r="A7" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="B7" t="s" s="9">
+      <c r="B7" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="11"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" t="s" s="8">
+      <c r="A8" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="B8" t="s" s="9">
+      <c r="B8" t="s" s="2">
         <v>11</v>
       </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="11"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" t="s" s="8">
+      <c r="A9" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="B9" t="s" s="9">
+      <c r="B9" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="11"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
     </row>
     <row r="10" ht="26.35" customHeight="1">
-      <c r="A10" t="s" s="8">
+      <c r="A10" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="B10" t="s" s="9">
+      <c r="B10" t="s" s="2">
         <v>15</v>
       </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="11"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
     </row>
     <row r="11" ht="26.35" customHeight="1">
-      <c r="A11" t="s" s="8">
+      <c r="A11" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="B11" t="s" s="9">
+      <c r="B11" t="s" s="2">
         <v>17</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="11"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" t="s" s="8">
+      <c r="A12" t="s" s="2">
         <v>18</v>
       </c>
-      <c r="B12" t="s" s="9">
+      <c r="B12" t="s" s="2">
         <v>19</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="11"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="4"/>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="4"/>
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" t="s" s="6">
+      <c r="A15" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="4"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" t="s" s="8">
+      <c r="A16" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="B16" t="s" s="8">
+      <c r="B16" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="C16" t="s" s="8">
+      <c r="C16" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="D16" t="s" s="8">
+      <c r="D16" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="E16" s="11"/>
+      <c r="E16" s="3"/>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" t="s" s="9">
+      <c r="A17" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B17" t="s" s="9">
+      <c r="B17" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C17" t="s" s="9">
+      <c r="C17" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D17" t="s" s="9">
+      <c r="D17" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="E17" s="11"/>
+      <c r="E17" s="3"/>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" t="s" s="9">
+      <c r="A18" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="B18" t="s" s="9">
+      <c r="B18" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C18" t="s" s="9">
+      <c r="C18" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D18" t="s" s="9">
+      <c r="D18" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="E18" s="11"/>
+      <c r="E18" s="3"/>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" t="s" s="9">
+      <c r="A19" t="s" s="2">
         <v>30</v>
       </c>
-      <c r="B19" t="s" s="9">
+      <c r="B19" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C19" t="s" s="9">
+      <c r="C19" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D19" t="s" s="9">
+      <c r="D19" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="E19" s="11"/>
+      <c r="E19" s="3"/>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" t="s" s="9">
+      <c r="A20" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="B20" t="s" s="9">
+      <c r="B20" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C20" t="s" s="9">
+      <c r="C20" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D20" t="s" s="9">
+      <c r="D20" t="s" s="2">
         <v>34</v>
       </c>
-      <c r="E20" s="11"/>
+      <c r="E20" s="3"/>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" t="s" s="9">
+      <c r="A21" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="B21" t="s" s="9">
+      <c r="B21" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C21" t="s" s="9">
+      <c r="C21" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D21" t="s" s="9">
+      <c r="D21" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="E21" s="11"/>
+      <c r="E21" s="3"/>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" t="s" s="9">
+      <c r="A22" t="s" s="2">
         <v>37</v>
       </c>
-      <c r="B22" t="s" s="9">
+      <c r="B22" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C22" t="s" s="9">
+      <c r="C22" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D22" t="s" s="9">
+      <c r="D22" t="s" s="2">
         <v>39</v>
       </c>
-      <c r="E22" s="11"/>
+      <c r="E22" s="3"/>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" t="s" s="9">
+      <c r="A23" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="B23" t="s" s="9">
+      <c r="B23" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C23" t="s" s="9">
+      <c r="C23" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D23" t="s" s="9">
+      <c r="D23" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="E23" s="11"/>
+      <c r="E23" s="3"/>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" t="s" s="9">
+      <c r="A24" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="B24" t="s" s="9">
+      <c r="B24" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C24" t="s" s="9">
+      <c r="C24" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D24" t="s" s="9">
+      <c r="D24" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="E24" s="11"/>
+      <c r="E24" s="3"/>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" t="s" s="9">
+      <c r="A25" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="B25" t="s" s="9">
+      <c r="B25" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C25" t="s" s="9">
+      <c r="C25" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D25" t="s" s="9">
+      <c r="D25" t="s" s="2">
         <v>45</v>
       </c>
-      <c r="E25" s="11"/>
+      <c r="E25" s="3"/>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" t="s" s="9">
+      <c r="A26" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="B26" t="s" s="9">
+      <c r="B26" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C26" t="s" s="9">
+      <c r="C26" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D26" t="s" s="9">
+      <c r="D26" t="s" s="2">
         <v>47</v>
       </c>
-      <c r="E26" s="11"/>
+      <c r="E26" s="3"/>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="A27" t="s" s="9">
+      <c r="A27" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B27" t="s" s="9">
+      <c r="B27" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C27" t="s" s="9">
+      <c r="C27" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D27" t="s" s="9">
+      <c r="D27" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="E27" s="11"/>
+      <c r="E27" s="3"/>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="A28" t="s" s="9">
+      <c r="A28" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="B28" t="s" s="9">
+      <c r="B28" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C28" t="s" s="9">
+      <c r="C28" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D28" t="s" s="9">
+      <c r="D28" t="s" s="2">
         <v>51</v>
       </c>
-      <c r="E28" s="11"/>
+      <c r="E28" s="3"/>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="A29" t="s" s="9">
+      <c r="A29" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="B29" t="s" s="9">
+      <c r="B29" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="C29" t="s" s="9">
+      <c r="C29" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D29" t="s" s="9">
+      <c r="D29" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="E29" s="11"/>
+      <c r="E29" s="3"/>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="A30" t="s" s="9">
+      <c r="A30" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="B30" t="s" s="9">
+      <c r="B30" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="C30" t="s" s="9">
+      <c r="C30" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D30" t="s" s="9">
+      <c r="D30" t="s" s="2">
         <v>56</v>
       </c>
-      <c r="E30" s="11"/>
+      <c r="E30" s="3"/>
     </row>
     <row r="31" ht="15" customHeight="1">
-      <c r="A31" t="s" s="9">
+      <c r="A31" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="B31" t="s" s="9">
+      <c r="B31" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C31" t="s" s="9">
+      <c r="C31" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D31" t="s" s="9">
+      <c r="D31" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="E31" s="11"/>
+      <c r="E31" s="3"/>
     </row>
     <row r="32" ht="15" customHeight="1">
-      <c r="A32" t="s" s="9">
+      <c r="A32" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="B32" t="s" s="9">
+      <c r="B32" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C32" t="s" s="9">
+      <c r="C32" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D32" t="s" s="9">
+      <c r="D32" t="s" s="2">
         <v>60</v>
       </c>
-      <c r="E32" s="11"/>
+      <c r="E32" s="3"/>
     </row>
     <row r="33" ht="15" customHeight="1">
-      <c r="A33" t="s" s="9">
+      <c r="A33" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B33" t="s" s="9">
+      <c r="B33" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C33" t="s" s="9">
+      <c r="C33" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D33" t="s" s="9">
+      <c r="D33" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="E33" s="11"/>
+      <c r="E33" s="3"/>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" t="s" s="9">
+      <c r="A34" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="B34" t="s" s="9">
+      <c r="B34" t="s" s="2">
         <v>64</v>
       </c>
-      <c r="C34" t="s" s="9">
+      <c r="C34" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D34" t="s" s="9">
+      <c r="D34" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="E34" s="11"/>
+      <c r="E34" s="3"/>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="A35" t="s" s="9">
+      <c r="A35" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="B35" t="s" s="9">
+      <c r="B35" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C35" t="s" s="9">
+      <c r="C35" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D35" t="s" s="9">
+      <c r="D35" t="s" s="2">
         <v>67</v>
       </c>
-      <c r="E35" s="11"/>
+      <c r="E35" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -3269,2957 +3146,2957 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:T51"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="16" style="13" customWidth="1"/>
-    <col min="2" max="2" width="14" style="13" customWidth="1"/>
-    <col min="3" max="4" width="18" style="13" customWidth="1"/>
-    <col min="5" max="6" width="12" style="13" customWidth="1"/>
-    <col min="7" max="7" width="24" style="13" customWidth="1"/>
-    <col min="8" max="8" width="34" style="13" customWidth="1"/>
-    <col min="9" max="11" width="14" style="13" customWidth="1"/>
-    <col min="12" max="12" width="34" style="13" customWidth="1"/>
-    <col min="13" max="13" width="15" style="13" customWidth="1"/>
-    <col min="14" max="14" width="14" style="13" customWidth="1"/>
-    <col min="15" max="16" width="20" style="13" customWidth="1"/>
-    <col min="17" max="17" width="24" style="13" customWidth="1"/>
-    <col min="18" max="18" width="18" style="13" customWidth="1"/>
-    <col min="19" max="19" width="50" style="13" customWidth="1"/>
-    <col min="20" max="20" width="8.85156" style="13" customWidth="1"/>
-    <col min="21" max="16384" width="8.85156" style="13" customWidth="1"/>
+    <col min="1" max="1" width="16" style="4" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
+    <col min="3" max="4" width="18" style="4" customWidth="1"/>
+    <col min="5" max="6" width="12" style="4" customWidth="1"/>
+    <col min="7" max="7" width="24" style="4" customWidth="1"/>
+    <col min="8" max="8" width="34" style="4" customWidth="1"/>
+    <col min="9" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="34" style="4" customWidth="1"/>
+    <col min="13" max="13" width="15" style="4" customWidth="1"/>
+    <col min="14" max="14" width="14" style="4" customWidth="1"/>
+    <col min="15" max="16" width="20" style="4" customWidth="1"/>
+    <col min="17" max="17" width="24" style="4" customWidth="1"/>
+    <col min="18" max="18" width="18" style="4" customWidth="1"/>
+    <col min="19" max="19" width="50" style="4" customWidth="1"/>
+    <col min="20" max="20" width="8.85156" style="4" customWidth="1"/>
+    <col min="21" max="16384" width="8.85156" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" t="s" s="14">
+      <c r="A1" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B1" t="s" s="14">
+      <c r="B1" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="C1" t="s" s="14">
+      <c r="C1" t="s" s="2">
         <v>30</v>
       </c>
-      <c r="D1" t="s" s="14">
+      <c r="D1" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="E1" t="s" s="14">
+      <c r="E1" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="F1" t="s" s="14">
+      <c r="F1" t="s" s="2">
         <v>37</v>
       </c>
-      <c r="G1" t="s" s="14">
+      <c r="G1" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="H1" t="s" s="14">
+      <c r="H1" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="I1" t="s" s="14">
+      <c r="I1" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="J1" t="s" s="14">
+      <c r="J1" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="K1" t="s" s="14">
+      <c r="K1" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="L1" t="s" s="14">
+      <c r="L1" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="M1" t="s" s="14">
+      <c r="M1" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="N1" t="s" s="14">
+      <c r="N1" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="O1" t="s" s="14">
+      <c r="O1" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="P1" t="s" s="14">
+      <c r="P1" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="Q1" t="s" s="14">
+      <c r="Q1" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="R1" t="s" s="14">
+      <c r="R1" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="S1" t="s" s="14">
+      <c r="S1" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="T1" s="11"/>
+      <c r="T1" s="3"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" t="s" s="15">
+      <c r="A2" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B2" t="s" s="15">
+      <c r="B2" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C2" t="s" s="15">
+      <c r="C2" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="D2" t="s" s="15">
+      <c r="D2" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="E2" t="s" s="15">
+      <c r="E2" t="s" s="2">
         <v>71</v>
       </c>
-      <c r="F2" t="s" s="15">
+      <c r="F2" t="s" s="2">
         <v>72</v>
       </c>
-      <c r="G2" t="s" s="15">
+      <c r="G2" t="s" s="2">
         <v>73</v>
       </c>
-      <c r="H2" t="s" s="15">
+      <c r="H2" t="s" s="2">
         <v>74</v>
       </c>
-      <c r="I2" t="s" s="15">
+      <c r="I2" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="J2" t="s" s="15">
+      <c r="J2" t="s" s="2">
         <v>76</v>
       </c>
-      <c r="K2" t="s" s="15">
+      <c r="K2" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L2" t="s" s="15">
+      <c r="L2" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M2" t="s" s="15">
+      <c r="M2" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N2" t="s" s="15">
+      <c r="N2" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O2" t="s" s="15">
+      <c r="O2" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="P2" t="s" s="15">
+      <c r="P2" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="Q2" t="s" s="15">
+      <c r="Q2" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R2" t="s" s="15">
+      <c r="R2" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S2" s="16"/>
-      <c r="T2" s="11"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" t="s" s="15">
+      <c r="A3" t="s" s="2">
         <v>85</v>
       </c>
-      <c r="B3" t="s" s="15">
+      <c r="B3" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C3" t="s" s="15">
+      <c r="C3" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="D3" t="s" s="15">
+      <c r="D3" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="E3" t="s" s="15">
+      <c r="E3" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F3" t="s" s="15">
+      <c r="F3" t="s" s="2">
         <v>88</v>
       </c>
-      <c r="G3" t="s" s="15">
+      <c r="G3" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H3" t="s" s="15">
+      <c r="H3" t="s" s="2">
         <v>90</v>
       </c>
-      <c r="I3" t="s" s="15">
+      <c r="I3" t="s" s="2">
         <v>91</v>
       </c>
-      <c r="J3" t="s" s="15">
+      <c r="J3" t="s" s="2">
         <v>92</v>
       </c>
-      <c r="K3" t="s" s="15">
+      <c r="K3" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L3" t="s" s="15">
+      <c r="L3" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M3" t="s" s="15">
+      <c r="M3" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N3" t="s" s="15">
+      <c r="N3" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O3" t="s" s="15">
+      <c r="O3" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="P3" t="s" s="15">
+      <c r="P3" t="s" s="2">
         <v>95</v>
       </c>
-      <c r="Q3" t="s" s="15">
+      <c r="Q3" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R3" t="s" s="15">
+      <c r="R3" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S3" s="16"/>
-      <c r="T3" s="11"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" t="s" s="15">
+      <c r="A4" t="s" s="2">
         <v>96</v>
       </c>
-      <c r="B4" t="s" s="15">
+      <c r="B4" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C4" t="s" s="15">
+      <c r="C4" t="s" s="2">
         <v>97</v>
       </c>
-      <c r="D4" t="s" s="15">
+      <c r="D4" t="s" s="2">
         <v>97</v>
       </c>
-      <c r="E4" t="s" s="15">
+      <c r="E4" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="F4" t="s" s="15">
+      <c r="F4" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="G4" t="s" s="15">
+      <c r="G4" t="s" s="2">
         <v>100</v>
       </c>
-      <c r="H4" t="s" s="15">
+      <c r="H4" t="s" s="2">
         <v>101</v>
       </c>
-      <c r="I4" t="s" s="15">
+      <c r="I4" t="s" s="2">
         <v>102</v>
       </c>
-      <c r="J4" t="s" s="15">
+      <c r="J4" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="K4" t="s" s="15">
+      <c r="K4" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L4" t="s" s="15">
+      <c r="L4" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M4" t="s" s="15">
+      <c r="M4" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N4" t="s" s="15">
+      <c r="N4" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O4" t="s" s="15">
+      <c r="O4" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="P4" t="s" s="15">
+      <c r="P4" t="s" s="2">
         <v>105</v>
       </c>
-      <c r="Q4" t="s" s="15">
+      <c r="Q4" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R4" t="s" s="15">
+      <c r="R4" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S4" s="16"/>
-      <c r="T4" s="11"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" t="s" s="15">
+      <c r="A5" t="s" s="2">
         <v>106</v>
       </c>
-      <c r="B5" t="s" s="15">
+      <c r="B5" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C5" t="s" s="15">
+      <c r="C5" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="D5" t="s" s="15">
+      <c r="D5" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="E5" t="s" s="15">
+      <c r="E5" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F5" t="s" s="15">
+      <c r="F5" t="s" s="2">
         <v>108</v>
       </c>
-      <c r="G5" t="s" s="15">
+      <c r="G5" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H5" t="s" s="15">
+      <c r="H5" t="s" s="2">
         <v>109</v>
       </c>
-      <c r="I5" t="s" s="15">
+      <c r="I5" t="s" s="2">
         <v>110</v>
       </c>
-      <c r="J5" t="s" s="15">
+      <c r="J5" t="s" s="2">
         <v>111</v>
       </c>
-      <c r="K5" t="s" s="15">
+      <c r="K5" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L5" t="s" s="15">
+      <c r="L5" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M5" t="s" s="15">
+      <c r="M5" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N5" t="s" s="15">
+      <c r="N5" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O5" t="s" s="15">
+      <c r="O5" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="P5" t="s" s="15">
+      <c r="P5" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="Q5" t="s" s="15">
+      <c r="Q5" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R5" t="s" s="15">
+      <c r="R5" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S5" s="16"/>
-      <c r="T5" s="11"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" t="s" s="15">
+      <c r="A6" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="B6" t="s" s="15">
+      <c r="B6" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C6" t="s" s="15">
+      <c r="C6" t="s" s="2">
         <v>115</v>
       </c>
-      <c r="D6" t="s" s="15">
+      <c r="D6" t="s" s="2">
         <v>115</v>
       </c>
-      <c r="E6" t="s" s="15">
+      <c r="E6" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F6" t="s" s="15">
+      <c r="F6" t="s" s="2">
         <v>116</v>
       </c>
-      <c r="G6" t="s" s="15">
+      <c r="G6" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H6" t="s" s="15">
+      <c r="H6" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="I6" t="s" s="15">
+      <c r="I6" t="s" s="2">
         <v>118</v>
       </c>
-      <c r="J6" t="s" s="15">
+      <c r="J6" t="s" s="2">
         <v>119</v>
       </c>
-      <c r="K6" t="s" s="15">
+      <c r="K6" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L6" t="s" s="15">
+      <c r="L6" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M6" t="s" s="15">
+      <c r="M6" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N6" t="s" s="15">
+      <c r="N6" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O6" t="s" s="15">
+      <c r="O6" t="s" s="2">
         <v>120</v>
       </c>
-      <c r="P6" t="s" s="15">
+      <c r="P6" t="s" s="2">
         <v>121</v>
       </c>
-      <c r="Q6" t="s" s="15">
+      <c r="Q6" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R6" t="s" s="15">
+      <c r="R6" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S6" s="16"/>
-      <c r="T6" s="11"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" t="s" s="15">
+      <c r="A7" t="s" s="2">
         <v>122</v>
       </c>
-      <c r="B7" t="s" s="15">
+      <c r="B7" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C7" t="s" s="15">
+      <c r="C7" t="s" s="2">
         <v>123</v>
       </c>
-      <c r="D7" t="s" s="15">
+      <c r="D7" t="s" s="2">
         <v>123</v>
       </c>
-      <c r="E7" t="s" s="15">
+      <c r="E7" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F7" t="s" s="15">
+      <c r="F7" t="s" s="2">
         <v>124</v>
       </c>
-      <c r="G7" t="s" s="15">
+      <c r="G7" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H7" t="s" s="15">
+      <c r="H7" t="s" s="2">
         <v>125</v>
       </c>
-      <c r="I7" t="s" s="15">
+      <c r="I7" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="J7" t="s" s="15">
+      <c r="J7" t="s" s="2">
         <v>127</v>
       </c>
-      <c r="K7" t="s" s="15">
+      <c r="K7" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L7" t="s" s="15">
+      <c r="L7" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M7" t="s" s="15">
+      <c r="M7" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N7" t="s" s="15">
+      <c r="N7" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O7" t="s" s="15">
+      <c r="O7" t="s" s="2">
         <v>128</v>
       </c>
-      <c r="P7" t="s" s="15">
+      <c r="P7" t="s" s="2">
         <v>129</v>
       </c>
-      <c r="Q7" t="s" s="15">
+      <c r="Q7" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R7" t="s" s="15">
+      <c r="R7" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S7" s="16"/>
-      <c r="T7" s="11"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" t="s" s="15">
+      <c r="A8" t="s" s="2">
         <v>130</v>
       </c>
-      <c r="B8" t="s" s="15">
+      <c r="B8" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C8" t="s" s="15">
+      <c r="C8" t="s" s="2">
         <v>131</v>
       </c>
-      <c r="D8" t="s" s="15">
+      <c r="D8" t="s" s="2">
         <v>131</v>
       </c>
-      <c r="E8" t="s" s="15">
+      <c r="E8" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F8" t="s" s="15">
+      <c r="F8" t="s" s="2">
         <v>132</v>
       </c>
-      <c r="G8" t="s" s="15">
+      <c r="G8" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H8" t="s" s="15">
+      <c r="H8" t="s" s="2">
         <v>133</v>
       </c>
-      <c r="I8" t="s" s="15">
+      <c r="I8" t="s" s="2">
         <v>134</v>
       </c>
-      <c r="J8" t="s" s="15">
+      <c r="J8" t="s" s="2">
         <v>135</v>
       </c>
-      <c r="K8" t="s" s="15">
+      <c r="K8" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L8" t="s" s="15">
+      <c r="L8" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M8" t="s" s="15">
+      <c r="M8" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N8" t="s" s="15">
+      <c r="N8" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O8" t="s" s="15">
+      <c r="O8" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="P8" t="s" s="15">
+      <c r="P8" t="s" s="2">
         <v>137</v>
       </c>
-      <c r="Q8" t="s" s="15">
+      <c r="Q8" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R8" t="s" s="15">
+      <c r="R8" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S8" s="16"/>
-      <c r="T8" s="11"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" t="s" s="15">
+      <c r="A9" t="s" s="2">
         <v>138</v>
       </c>
-      <c r="B9" t="s" s="15">
+      <c r="B9" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C9" t="s" s="15">
+      <c r="C9" t="s" s="2">
         <v>139</v>
       </c>
-      <c r="D9" t="s" s="15">
+      <c r="D9" t="s" s="2">
         <v>139</v>
       </c>
-      <c r="E9" t="s" s="15">
+      <c r="E9" t="s" s="2">
         <v>140</v>
       </c>
-      <c r="F9" t="s" s="15">
+      <c r="F9" t="s" s="2">
         <v>141</v>
       </c>
-      <c r="G9" t="s" s="15">
+      <c r="G9" t="s" s="2">
         <v>142</v>
       </c>
-      <c r="H9" t="s" s="15">
+      <c r="H9" t="s" s="2">
         <v>143</v>
       </c>
-      <c r="I9" t="s" s="15">
+      <c r="I9" t="s" s="2">
         <v>144</v>
       </c>
-      <c r="J9" t="s" s="15">
+      <c r="J9" t="s" s="2">
         <v>145</v>
       </c>
-      <c r="K9" t="s" s="15">
+      <c r="K9" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L9" t="s" s="15">
+      <c r="L9" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M9" t="s" s="15">
+      <c r="M9" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N9" t="s" s="15">
+      <c r="N9" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O9" t="s" s="15">
+      <c r="O9" t="s" s="2">
         <v>146</v>
       </c>
-      <c r="P9" t="s" s="15">
+      <c r="P9" t="s" s="2">
         <v>147</v>
       </c>
-      <c r="Q9" t="s" s="15">
+      <c r="Q9" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R9" t="s" s="15">
+      <c r="R9" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S9" s="16"/>
-      <c r="T9" s="11"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" t="s" s="15">
+      <c r="A10" t="s" s="2">
         <v>148</v>
       </c>
-      <c r="B10" t="s" s="15">
+      <c r="B10" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C10" t="s" s="15">
+      <c r="C10" t="s" s="2">
         <v>149</v>
       </c>
-      <c r="D10" t="s" s="15">
+      <c r="D10" t="s" s="2">
         <v>149</v>
       </c>
-      <c r="E10" t="s" s="15">
+      <c r="E10" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F10" t="s" s="15">
+      <c r="F10" t="s" s="2">
         <v>150</v>
       </c>
-      <c r="G10" t="s" s="15">
+      <c r="G10" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H10" t="s" s="15">
+      <c r="H10" t="s" s="2">
         <v>151</v>
       </c>
-      <c r="I10" t="s" s="15">
+      <c r="I10" t="s" s="2">
         <v>152</v>
       </c>
-      <c r="J10" t="s" s="15">
+      <c r="J10" t="s" s="2">
         <v>153</v>
       </c>
-      <c r="K10" t="s" s="15">
+      <c r="K10" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L10" t="s" s="15">
+      <c r="L10" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M10" t="s" s="15">
+      <c r="M10" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N10" t="s" s="15">
+      <c r="N10" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O10" t="s" s="15">
+      <c r="O10" t="s" s="2">
         <v>154</v>
       </c>
-      <c r="P10" t="s" s="15">
+      <c r="P10" t="s" s="2">
         <v>155</v>
       </c>
-      <c r="Q10" t="s" s="15">
+      <c r="Q10" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R10" t="s" s="15">
+      <c r="R10" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S10" s="16"/>
-      <c r="T10" s="11"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" t="s" s="15">
+      <c r="A11" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="B11" t="s" s="15">
+      <c r="B11" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C11" t="s" s="15">
+      <c r="C11" t="s" s="2">
         <v>157</v>
       </c>
-      <c r="D11" t="s" s="15">
+      <c r="D11" t="s" s="2">
         <v>157</v>
       </c>
-      <c r="E11" t="s" s="15">
+      <c r="E11" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F11" t="s" s="15">
+      <c r="F11" t="s" s="2">
         <v>158</v>
       </c>
-      <c r="G11" t="s" s="15">
+      <c r="G11" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H11" t="s" s="15">
+      <c r="H11" t="s" s="2">
         <v>159</v>
       </c>
-      <c r="I11" t="s" s="15">
+      <c r="I11" t="s" s="2">
         <v>160</v>
       </c>
-      <c r="J11" t="s" s="15">
+      <c r="J11" t="s" s="2">
         <v>161</v>
       </c>
-      <c r="K11" t="s" s="15">
+      <c r="K11" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L11" t="s" s="15">
+      <c r="L11" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M11" t="s" s="15">
+      <c r="M11" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N11" t="s" s="15">
+      <c r="N11" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O11" t="s" s="15">
+      <c r="O11" t="s" s="2">
         <v>162</v>
       </c>
-      <c r="P11" t="s" s="15">
+      <c r="P11" t="s" s="2">
         <v>163</v>
       </c>
-      <c r="Q11" t="s" s="15">
+      <c r="Q11" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R11" t="s" s="15">
+      <c r="R11" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S11" s="16"/>
-      <c r="T11" s="11"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" t="s" s="15">
+      <c r="A12" t="s" s="2">
         <v>164</v>
       </c>
-      <c r="B12" t="s" s="15">
+      <c r="B12" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C12" t="s" s="15">
+      <c r="C12" t="s" s="2">
         <v>165</v>
       </c>
-      <c r="D12" t="s" s="15">
+      <c r="D12" t="s" s="2">
         <v>165</v>
       </c>
-      <c r="E12" t="s" s="15">
+      <c r="E12" t="s" s="2">
         <v>166</v>
       </c>
-      <c r="F12" t="s" s="15">
+      <c r="F12" t="s" s="2">
         <v>167</v>
       </c>
-      <c r="G12" t="s" s="15">
+      <c r="G12" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="H12" t="s" s="15">
+      <c r="H12" t="s" s="2">
         <v>169</v>
       </c>
-      <c r="I12" t="s" s="15">
+      <c r="I12" t="s" s="2">
         <v>170</v>
       </c>
-      <c r="J12" t="s" s="15">
+      <c r="J12" t="s" s="2">
         <v>171</v>
       </c>
-      <c r="K12" t="s" s="15">
+      <c r="K12" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L12" t="s" s="15">
+      <c r="L12" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M12" t="s" s="15">
+      <c r="M12" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N12" t="s" s="15">
+      <c r="N12" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O12" t="s" s="15">
+      <c r="O12" t="s" s="2">
         <v>172</v>
       </c>
-      <c r="P12" t="s" s="15">
+      <c r="P12" t="s" s="2">
         <v>173</v>
       </c>
-      <c r="Q12" t="s" s="15">
+      <c r="Q12" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R12" t="s" s="15">
+      <c r="R12" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S12" s="16"/>
-      <c r="T12" s="11"/>
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" t="s" s="15">
+      <c r="A13" t="s" s="2">
         <v>174</v>
       </c>
-      <c r="B13" t="s" s="15">
+      <c r="B13" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C13" t="s" s="15">
+      <c r="C13" t="s" s="2">
         <v>175</v>
       </c>
-      <c r="D13" t="s" s="15">
+      <c r="D13" t="s" s="2">
         <v>175</v>
       </c>
-      <c r="E13" t="s" s="15">
+      <c r="E13" t="s" s="2">
         <v>166</v>
       </c>
-      <c r="F13" t="s" s="15">
+      <c r="F13" t="s" s="2">
         <v>176</v>
       </c>
-      <c r="G13" t="s" s="15">
+      <c r="G13" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="H13" t="s" s="15">
+      <c r="H13" t="s" s="2">
         <v>177</v>
       </c>
-      <c r="I13" t="s" s="15">
+      <c r="I13" t="s" s="2">
         <v>178</v>
       </c>
-      <c r="J13" t="s" s="15">
+      <c r="J13" t="s" s="2">
         <v>179</v>
       </c>
-      <c r="K13" t="s" s="15">
+      <c r="K13" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L13" t="s" s="15">
+      <c r="L13" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M13" t="s" s="15">
+      <c r="M13" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N13" t="s" s="15">
+      <c r="N13" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O13" t="s" s="15">
+      <c r="O13" t="s" s="2">
         <v>128</v>
       </c>
-      <c r="P13" t="s" s="15">
+      <c r="P13" t="s" s="2">
         <v>180</v>
       </c>
-      <c r="Q13" t="s" s="15">
+      <c r="Q13" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R13" t="s" s="15">
+      <c r="R13" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S13" s="16"/>
-      <c r="T13" s="11"/>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" t="s" s="15">
+      <c r="A14" t="s" s="2">
         <v>181</v>
       </c>
-      <c r="B14" t="s" s="15">
+      <c r="B14" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C14" t="s" s="15">
+      <c r="C14" t="s" s="2">
         <v>182</v>
       </c>
-      <c r="D14" t="s" s="15">
+      <c r="D14" t="s" s="2">
         <v>182</v>
       </c>
-      <c r="E14" t="s" s="15">
+      <c r="E14" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F14" t="s" s="15">
+      <c r="F14" t="s" s="2">
         <v>183</v>
       </c>
-      <c r="G14" t="s" s="15">
+      <c r="G14" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H14" t="s" s="15">
+      <c r="H14" t="s" s="2">
         <v>184</v>
       </c>
-      <c r="I14" t="s" s="15">
+      <c r="I14" t="s" s="2">
         <v>185</v>
       </c>
-      <c r="J14" t="s" s="15">
+      <c r="J14" t="s" s="2">
         <v>186</v>
       </c>
-      <c r="K14" t="s" s="15">
+      <c r="K14" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L14" t="s" s="15">
+      <c r="L14" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M14" t="s" s="15">
+      <c r="M14" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N14" t="s" s="15">
+      <c r="N14" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O14" t="s" s="15">
+      <c r="O14" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="P14" t="s" s="15">
+      <c r="P14" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="Q14" t="s" s="15">
+      <c r="Q14" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R14" t="s" s="15">
+      <c r="R14" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S14" s="16"/>
-      <c r="T14" s="11"/>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" t="s" s="15">
+      <c r="A15" t="s" s="2">
         <v>187</v>
       </c>
-      <c r="B15" t="s" s="15">
+      <c r="B15" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C15" t="s" s="15">
+      <c r="C15" t="s" s="2">
         <v>188</v>
       </c>
-      <c r="D15" t="s" s="15">
+      <c r="D15" t="s" s="2">
         <v>188</v>
       </c>
-      <c r="E15" t="s" s="15">
+      <c r="E15" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F15" t="s" s="15">
+      <c r="F15" t="s" s="2">
         <v>189</v>
       </c>
-      <c r="G15" t="s" s="15">
+      <c r="G15" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H15" t="s" s="15">
+      <c r="H15" t="s" s="2">
         <v>190</v>
       </c>
-      <c r="I15" t="s" s="15">
+      <c r="I15" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="J15" t="s" s="15">
+      <c r="J15" t="s" s="2">
         <v>192</v>
       </c>
-      <c r="K15" t="s" s="15">
+      <c r="K15" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L15" t="s" s="15">
+      <c r="L15" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M15" t="s" s="15">
+      <c r="M15" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N15" t="s" s="15">
+      <c r="N15" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O15" t="s" s="15">
+      <c r="O15" t="s" s="2">
         <v>193</v>
       </c>
-      <c r="P15" t="s" s="15">
+      <c r="P15" t="s" s="2">
         <v>194</v>
       </c>
-      <c r="Q15" t="s" s="15">
+      <c r="Q15" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R15" t="s" s="15">
+      <c r="R15" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S15" s="16"/>
-      <c r="T15" s="11"/>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" t="s" s="15">
+      <c r="A16" t="s" s="2">
         <v>195</v>
       </c>
-      <c r="B16" t="s" s="15">
+      <c r="B16" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C16" t="s" s="15">
+      <c r="C16" t="s" s="2">
         <v>196</v>
       </c>
-      <c r="D16" t="s" s="15">
+      <c r="D16" t="s" s="2">
         <v>196</v>
       </c>
-      <c r="E16" t="s" s="15">
+      <c r="E16" t="s" s="2">
         <v>71</v>
       </c>
-      <c r="F16" t="s" s="15">
+      <c r="F16" t="s" s="2">
         <v>197</v>
       </c>
-      <c r="G16" t="s" s="15">
+      <c r="G16" t="s" s="2">
         <v>198</v>
       </c>
-      <c r="H16" t="s" s="15">
+      <c r="H16" t="s" s="2">
         <v>199</v>
       </c>
-      <c r="I16" t="s" s="15">
+      <c r="I16" t="s" s="2">
         <v>200</v>
       </c>
-      <c r="J16" t="s" s="15">
+      <c r="J16" t="s" s="2">
         <v>201</v>
       </c>
-      <c r="K16" t="s" s="15">
+      <c r="K16" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L16" t="s" s="15">
+      <c r="L16" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M16" t="s" s="15">
+      <c r="M16" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N16" t="s" s="15">
+      <c r="N16" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O16" t="s" s="15">
+      <c r="O16" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="P16" t="s" s="15">
+      <c r="P16" t="s" s="2">
         <v>202</v>
       </c>
-      <c r="Q16" t="s" s="15">
+      <c r="Q16" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R16" t="s" s="15">
+      <c r="R16" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S16" s="16"/>
-      <c r="T16" s="11"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" t="s" s="15">
+      <c r="A17" t="s" s="2">
         <v>203</v>
       </c>
-      <c r="B17" t="s" s="15">
+      <c r="B17" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C17" t="s" s="15">
+      <c r="C17" t="s" s="2">
         <v>204</v>
       </c>
-      <c r="D17" t="s" s="15">
+      <c r="D17" t="s" s="2">
         <v>204</v>
       </c>
-      <c r="E17" t="s" s="15">
+      <c r="E17" t="s" s="2">
         <v>205</v>
       </c>
-      <c r="F17" t="s" s="15">
+      <c r="F17" t="s" s="2">
         <v>206</v>
       </c>
-      <c r="G17" t="s" s="15">
+      <c r="G17" t="s" s="2">
         <v>207</v>
       </c>
-      <c r="H17" t="s" s="15">
+      <c r="H17" t="s" s="2">
         <v>208</v>
       </c>
-      <c r="I17" t="s" s="15">
+      <c r="I17" t="s" s="2">
         <v>209</v>
       </c>
-      <c r="J17" t="s" s="15">
+      <c r="J17" t="s" s="2">
         <v>210</v>
       </c>
-      <c r="K17" t="s" s="15">
+      <c r="K17" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L17" t="s" s="15">
+      <c r="L17" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M17" t="s" s="15">
+      <c r="M17" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N17" t="s" s="15">
+      <c r="N17" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O17" t="s" s="15">
+      <c r="O17" t="s" s="2">
         <v>211</v>
       </c>
-      <c r="P17" t="s" s="15">
+      <c r="P17" t="s" s="2">
         <v>194</v>
       </c>
-      <c r="Q17" t="s" s="15">
+      <c r="Q17" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R17" t="s" s="15">
+      <c r="R17" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S17" s="16"/>
-      <c r="T17" s="11"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" t="s" s="15">
+      <c r="A18" t="s" s="2">
         <v>212</v>
       </c>
-      <c r="B18" t="s" s="15">
+      <c r="B18" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C18" t="s" s="15">
+      <c r="C18" t="s" s="2">
         <v>213</v>
       </c>
-      <c r="D18" t="s" s="15">
+      <c r="D18" t="s" s="2">
         <v>213</v>
       </c>
-      <c r="E18" t="s" s="15">
+      <c r="E18" t="s" s="2">
         <v>166</v>
       </c>
-      <c r="F18" t="s" s="15">
+      <c r="F18" t="s" s="2">
         <v>214</v>
       </c>
-      <c r="G18" t="s" s="15">
+      <c r="G18" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="H18" t="s" s="15">
+      <c r="H18" t="s" s="2">
         <v>215</v>
       </c>
-      <c r="I18" t="s" s="15">
+      <c r="I18" t="s" s="2">
         <v>216</v>
       </c>
-      <c r="J18" t="s" s="15">
+      <c r="J18" t="s" s="2">
         <v>217</v>
       </c>
-      <c r="K18" t="s" s="15">
+      <c r="K18" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L18" t="s" s="15">
+      <c r="L18" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M18" t="s" s="15">
+      <c r="M18" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N18" t="s" s="15">
+      <c r="N18" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O18" t="s" s="15">
+      <c r="O18" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="P18" t="s" s="15">
+      <c r="P18" t="s" s="2">
         <v>218</v>
       </c>
-      <c r="Q18" t="s" s="15">
+      <c r="Q18" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R18" t="s" s="15">
+      <c r="R18" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S18" s="16"/>
-      <c r="T18" s="11"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" t="s" s="15">
+      <c r="A19" t="s" s="2">
         <v>219</v>
       </c>
-      <c r="B19" t="s" s="15">
+      <c r="B19" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C19" t="s" s="15">
+      <c r="C19" t="s" s="2">
         <v>221</v>
       </c>
-      <c r="D19" t="s" s="15">
+      <c r="D19" t="s" s="2">
         <v>221</v>
       </c>
-      <c r="E19" t="s" s="15">
+      <c r="E19" t="s" s="2">
         <v>222</v>
       </c>
-      <c r="F19" t="s" s="15">
+      <c r="F19" t="s" s="2">
         <v>223</v>
       </c>
-      <c r="G19" t="s" s="15">
+      <c r="G19" t="s" s="2">
         <v>224</v>
       </c>
-      <c r="H19" t="s" s="15">
+      <c r="H19" t="s" s="2">
         <v>225</v>
       </c>
-      <c r="I19" t="s" s="15">
+      <c r="I19" t="s" s="2">
         <v>226</v>
       </c>
-      <c r="J19" t="s" s="15">
+      <c r="J19" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="K19" t="s" s="15">
+      <c r="K19" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L19" t="s" s="15">
+      <c r="L19" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M19" t="s" s="15">
+      <c r="M19" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N19" t="s" s="15">
+      <c r="N19" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O19" t="s" s="15">
+      <c r="O19" t="s" s="2">
         <v>228</v>
       </c>
-      <c r="P19" t="s" s="15">
+      <c r="P19" t="s" s="2">
         <v>229</v>
       </c>
-      <c r="Q19" t="s" s="15">
+      <c r="Q19" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R19" t="s" s="15">
+      <c r="R19" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S19" s="16"/>
-      <c r="T19" s="11"/>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" t="s" s="15">
+      <c r="A20" t="s" s="2">
         <v>230</v>
       </c>
-      <c r="B20" t="s" s="15">
+      <c r="B20" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C20" t="s" s="15">
+      <c r="C20" t="s" s="2">
         <v>231</v>
       </c>
-      <c r="D20" t="s" s="15">
+      <c r="D20" t="s" s="2">
         <v>231</v>
       </c>
-      <c r="E20" t="s" s="15">
+      <c r="E20" t="s" s="2">
         <v>232</v>
       </c>
-      <c r="F20" t="s" s="15">
+      <c r="F20" t="s" s="2">
         <v>233</v>
       </c>
-      <c r="G20" t="s" s="15">
+      <c r="G20" t="s" s="2">
         <v>234</v>
       </c>
-      <c r="H20" t="s" s="15">
+      <c r="H20" t="s" s="2">
         <v>235</v>
       </c>
-      <c r="I20" t="s" s="15">
+      <c r="I20" t="s" s="2">
         <v>236</v>
       </c>
-      <c r="J20" t="s" s="15">
+      <c r="J20" t="s" s="2">
         <v>237</v>
       </c>
-      <c r="K20" t="s" s="15">
+      <c r="K20" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L20" t="s" s="15">
+      <c r="L20" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M20" t="s" s="15">
+      <c r="M20" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N20" t="s" s="15">
+      <c r="N20" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O20" t="s" s="15">
+      <c r="O20" t="s" s="2">
         <v>238</v>
       </c>
-      <c r="P20" t="s" s="15">
+      <c r="P20" t="s" s="2">
         <v>218</v>
       </c>
-      <c r="Q20" t="s" s="15">
+      <c r="Q20" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R20" t="s" s="15">
+      <c r="R20" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S20" s="16"/>
-      <c r="T20" s="11"/>
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" t="s" s="15">
+      <c r="A21" t="s" s="2">
         <v>239</v>
       </c>
-      <c r="B21" t="s" s="15">
+      <c r="B21" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C21" t="s" s="15">
+      <c r="C21" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="D21" t="s" s="15">
+      <c r="D21" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="E21" t="s" s="15">
+      <c r="E21" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="F21" t="s" s="15">
+      <c r="F21" t="s" s="2">
         <v>242</v>
       </c>
-      <c r="G21" t="s" s="15">
+      <c r="G21" t="s" s="2">
         <v>243</v>
       </c>
-      <c r="H21" t="s" s="15">
+      <c r="H21" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="I21" t="s" s="15">
+      <c r="I21" t="s" s="2">
         <v>245</v>
       </c>
-      <c r="J21" t="s" s="15">
+      <c r="J21" t="s" s="2">
         <v>246</v>
       </c>
-      <c r="K21" t="s" s="15">
+      <c r="K21" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L21" t="s" s="15">
+      <c r="L21" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M21" t="s" s="15">
+      <c r="M21" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N21" t="s" s="15">
+      <c r="N21" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O21" t="s" s="15">
+      <c r="O21" t="s" s="2">
         <v>202</v>
       </c>
-      <c r="P21" t="s" s="15">
+      <c r="P21" t="s" s="2">
         <v>247</v>
       </c>
-      <c r="Q21" t="s" s="15">
+      <c r="Q21" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R21" t="s" s="15">
+      <c r="R21" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S21" s="16"/>
-      <c r="T21" s="11"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" t="s" s="15">
+      <c r="A22" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="B22" t="s" s="15">
+      <c r="B22" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C22" t="s" s="15">
+      <c r="C22" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="D22" t="s" s="15">
+      <c r="D22" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="E22" t="s" s="15">
+      <c r="E22" t="s" s="2">
         <v>250</v>
       </c>
-      <c r="F22" t="s" s="15">
+      <c r="F22" t="s" s="2">
         <v>251</v>
       </c>
-      <c r="G22" t="s" s="15">
+      <c r="G22" t="s" s="2">
         <v>252</v>
       </c>
-      <c r="H22" t="s" s="15">
+      <c r="H22" t="s" s="2">
         <v>253</v>
       </c>
-      <c r="I22" t="s" s="15">
+      <c r="I22" t="s" s="2">
         <v>254</v>
       </c>
-      <c r="J22" t="s" s="15">
+      <c r="J22" t="s" s="2">
         <v>255</v>
       </c>
-      <c r="K22" t="s" s="15">
+      <c r="K22" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L22" t="s" s="15">
+      <c r="L22" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M22" t="s" s="15">
+      <c r="M22" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N22" t="s" s="15">
+      <c r="N22" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O22" s="17">
+      <c r="O22" s="5">
         <v>87</v>
       </c>
-      <c r="P22" s="17">
+      <c r="P22" s="5">
         <v>17.3333333333333</v>
       </c>
-      <c r="Q22" t="s" s="15">
+      <c r="Q22" t="s" s="2">
         <v>256</v>
       </c>
-      <c r="R22" t="s" s="15">
+      <c r="R22" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S22" t="s" s="15">
+      <c r="S22" t="s" s="2">
         <v>257</v>
       </c>
-      <c r="T22" s="11"/>
+      <c r="T22" s="3"/>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" t="s" s="15">
+      <c r="A23" t="s" s="2">
         <v>258</v>
       </c>
-      <c r="B23" t="s" s="15">
+      <c r="B23" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C23" t="s" s="15">
+      <c r="C23" t="s" s="2">
         <v>259</v>
       </c>
-      <c r="D23" t="s" s="15">
+      <c r="D23" t="s" s="2">
         <v>259</v>
       </c>
-      <c r="E23" t="s" s="15">
+      <c r="E23" t="s" s="2">
         <v>260</v>
       </c>
-      <c r="F23" t="s" s="15">
+      <c r="F23" t="s" s="2">
         <v>261</v>
       </c>
-      <c r="G23" t="s" s="15">
+      <c r="G23" t="s" s="2">
         <v>262</v>
       </c>
-      <c r="H23" t="s" s="15">
+      <c r="H23" t="s" s="2">
         <v>263</v>
       </c>
-      <c r="I23" t="s" s="15">
+      <c r="I23" t="s" s="2">
         <v>264</v>
       </c>
-      <c r="J23" t="s" s="15">
+      <c r="J23" t="s" s="2">
         <v>265</v>
       </c>
-      <c r="K23" t="s" s="15">
+      <c r="K23" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L23" t="s" s="15">
+      <c r="L23" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M23" t="s" s="15">
+      <c r="M23" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N23" t="s" s="15">
+      <c r="N23" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O23" t="s" s="15">
+      <c r="O23" t="s" s="2">
         <v>266</v>
       </c>
-      <c r="P23" t="s" s="15">
+      <c r="P23" t="s" s="2">
         <v>266</v>
       </c>
-      <c r="Q23" t="s" s="15">
+      <c r="Q23" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R23" t="s" s="15">
+      <c r="R23" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S23" s="16"/>
-      <c r="T23" s="11"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" t="s" s="15">
+      <c r="A24" t="s" s="2">
         <v>267</v>
       </c>
-      <c r="B24" t="s" s="15">
+      <c r="B24" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C24" t="s" s="15">
+      <c r="C24" t="s" s="2">
         <v>268</v>
       </c>
-      <c r="D24" t="s" s="15">
+      <c r="D24" t="s" s="2">
         <v>268</v>
       </c>
-      <c r="E24" t="s" s="15">
+      <c r="E24" t="s" s="2">
         <v>269</v>
       </c>
-      <c r="F24" t="s" s="15">
+      <c r="F24" t="s" s="2">
         <v>270</v>
       </c>
-      <c r="G24" t="s" s="15">
+      <c r="G24" t="s" s="2">
         <v>271</v>
       </c>
-      <c r="H24" t="s" s="15">
+      <c r="H24" t="s" s="2">
         <v>272</v>
       </c>
-      <c r="I24" t="s" s="15">
+      <c r="I24" t="s" s="2">
         <v>273</v>
       </c>
-      <c r="J24" t="s" s="15">
+      <c r="J24" t="s" s="2">
         <v>274</v>
       </c>
-      <c r="K24" t="s" s="15">
+      <c r="K24" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L24" t="s" s="15">
+      <c r="L24" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M24" t="s" s="15">
+      <c r="M24" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N24" t="s" s="15">
+      <c r="N24" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O24" t="s" s="15">
+      <c r="O24" t="s" s="2">
         <v>275</v>
       </c>
-      <c r="P24" t="s" s="15">
+      <c r="P24" t="s" s="2">
         <v>276</v>
       </c>
-      <c r="Q24" t="s" s="15">
+      <c r="Q24" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R24" t="s" s="15">
+      <c r="R24" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S24" s="16"/>
-      <c r="T24" s="11"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" t="s" s="15">
+      <c r="A25" t="s" s="2">
         <v>277</v>
       </c>
-      <c r="B25" t="s" s="15">
+      <c r="B25" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C25" t="s" s="15">
+      <c r="C25" t="s" s="2">
         <v>278</v>
       </c>
-      <c r="D25" t="s" s="15">
+      <c r="D25" t="s" s="2">
         <v>278</v>
       </c>
-      <c r="E25" t="s" s="15">
+      <c r="E25" t="s" s="2">
         <v>279</v>
       </c>
-      <c r="F25" t="s" s="15">
+      <c r="F25" t="s" s="2">
         <v>280</v>
       </c>
-      <c r="G25" t="s" s="15">
+      <c r="G25" t="s" s="2">
         <v>281</v>
       </c>
-      <c r="H25" t="s" s="15">
+      <c r="H25" t="s" s="2">
         <v>282</v>
       </c>
-      <c r="I25" t="s" s="15">
+      <c r="I25" t="s" s="2">
         <v>283</v>
       </c>
-      <c r="J25" t="s" s="15">
+      <c r="J25" t="s" s="2">
         <v>284</v>
       </c>
-      <c r="K25" t="s" s="15">
+      <c r="K25" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L25" t="s" s="15">
+      <c r="L25" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M25" t="s" s="15">
+      <c r="M25" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N25" t="s" s="15">
+      <c r="N25" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O25" t="s" s="15">
+      <c r="O25" t="s" s="2">
         <v>285</v>
       </c>
-      <c r="P25" t="s" s="15">
+      <c r="P25" t="s" s="2">
         <v>286</v>
       </c>
-      <c r="Q25" t="s" s="15">
+      <c r="Q25" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R25" t="s" s="15">
+      <c r="R25" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S25" s="16"/>
-      <c r="T25" s="11"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" t="s" s="15">
+      <c r="A26" t="s" s="2">
         <v>287</v>
       </c>
-      <c r="B26" t="s" s="15">
+      <c r="B26" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C26" t="s" s="15">
+      <c r="C26" t="s" s="2">
         <v>289</v>
       </c>
-      <c r="D26" t="s" s="15">
+      <c r="D26" t="s" s="2">
         <v>289</v>
       </c>
-      <c r="E26" t="s" s="15">
+      <c r="E26" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="F26" t="s" s="15">
+      <c r="F26" t="s" s="2">
         <v>291</v>
       </c>
-      <c r="G26" t="s" s="15">
+      <c r="G26" t="s" s="2">
         <v>292</v>
       </c>
-      <c r="H26" t="s" s="15">
+      <c r="H26" t="s" s="2">
         <v>293</v>
       </c>
-      <c r="I26" t="s" s="15">
+      <c r="I26" t="s" s="2">
         <v>294</v>
       </c>
-      <c r="J26" t="s" s="15">
+      <c r="J26" t="s" s="2">
         <v>295</v>
       </c>
-      <c r="K26" t="s" s="15">
+      <c r="K26" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L26" t="s" s="15">
+      <c r="L26" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M26" t="s" s="15">
+      <c r="M26" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N26" t="s" s="15">
+      <c r="N26" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O26" t="s" s="15">
+      <c r="O26" t="s" s="2">
         <v>296</v>
       </c>
-      <c r="P26" t="s" s="15">
+      <c r="P26" t="s" s="2">
         <v>297</v>
       </c>
-      <c r="Q26" t="s" s="15">
+      <c r="Q26" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R26" t="s" s="15">
+      <c r="R26" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S26" s="16"/>
-      <c r="T26" s="11"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" t="s" s="15">
+      <c r="A27" t="s" s="2">
         <v>298</v>
       </c>
-      <c r="B27" t="s" s="15">
+      <c r="B27" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C27" t="s" s="15">
+      <c r="C27" t="s" s="2">
         <v>299</v>
       </c>
-      <c r="D27" t="s" s="15">
+      <c r="D27" t="s" s="2">
         <v>299</v>
       </c>
-      <c r="E27" t="s" s="15">
+      <c r="E27" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="F27" t="s" s="15">
+      <c r="F27" t="s" s="2">
         <v>300</v>
       </c>
-      <c r="G27" t="s" s="15">
+      <c r="G27" t="s" s="2">
         <v>292</v>
       </c>
-      <c r="H27" t="s" s="15">
+      <c r="H27" t="s" s="2">
         <v>301</v>
       </c>
-      <c r="I27" t="s" s="15">
+      <c r="I27" t="s" s="2">
         <v>302</v>
       </c>
-      <c r="J27" t="s" s="15">
+      <c r="J27" t="s" s="2">
         <v>303</v>
       </c>
-      <c r="K27" t="s" s="15">
+      <c r="K27" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L27" t="s" s="15">
+      <c r="L27" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M27" t="s" s="15">
+      <c r="M27" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N27" t="s" s="15">
+      <c r="N27" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O27" t="s" s="15">
+      <c r="O27" t="s" s="2">
         <v>304</v>
       </c>
-      <c r="P27" t="s" s="15">
+      <c r="P27" t="s" s="2">
         <v>238</v>
       </c>
-      <c r="Q27" t="s" s="15">
+      <c r="Q27" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R27" t="s" s="15">
+      <c r="R27" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S27" s="16"/>
-      <c r="T27" s="11"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" t="s" s="15">
+      <c r="A28" t="s" s="2">
         <v>305</v>
       </c>
-      <c r="B28" t="s" s="15">
+      <c r="B28" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C28" t="s" s="15">
+      <c r="C28" t="s" s="2">
         <v>306</v>
       </c>
-      <c r="D28" t="s" s="15">
+      <c r="D28" t="s" s="2">
         <v>306</v>
       </c>
-      <c r="E28" t="s" s="15">
+      <c r="E28" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="F28" t="s" s="15">
+      <c r="F28" t="s" s="2">
         <v>308</v>
       </c>
-      <c r="G28" t="s" s="15">
+      <c r="G28" t="s" s="2">
         <v>309</v>
       </c>
-      <c r="H28" t="s" s="15">
+      <c r="H28" t="s" s="2">
         <v>310</v>
       </c>
-      <c r="I28" t="s" s="15">
+      <c r="I28" t="s" s="2">
         <v>311</v>
       </c>
-      <c r="J28" t="s" s="15">
+      <c r="J28" t="s" s="2">
         <v>312</v>
       </c>
-      <c r="K28" t="s" s="15">
+      <c r="K28" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L28" t="s" s="15">
+      <c r="L28" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M28" t="s" s="15">
+      <c r="M28" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N28" t="s" s="15">
+      <c r="N28" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O28" t="s" s="15">
+      <c r="O28" t="s" s="2">
         <v>313</v>
       </c>
-      <c r="P28" t="s" s="15">
+      <c r="P28" t="s" s="2">
         <v>314</v>
       </c>
-      <c r="Q28" t="s" s="15">
+      <c r="Q28" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R28" t="s" s="15">
+      <c r="R28" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S28" s="16"/>
-      <c r="T28" s="11"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" t="s" s="15">
+      <c r="A29" t="s" s="2">
         <v>315</v>
       </c>
-      <c r="B29" t="s" s="15">
+      <c r="B29" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C29" t="s" s="15">
+      <c r="C29" t="s" s="2">
         <v>316</v>
       </c>
-      <c r="D29" t="s" s="15">
+      <c r="D29" t="s" s="2">
         <v>317</v>
       </c>
-      <c r="E29" t="s" s="15">
+      <c r="E29" t="s" s="2">
         <v>318</v>
       </c>
-      <c r="F29" t="s" s="15">
+      <c r="F29" t="s" s="2">
         <v>319</v>
       </c>
-      <c r="G29" t="s" s="15">
+      <c r="G29" t="s" s="2">
         <v>320</v>
       </c>
-      <c r="H29" t="s" s="15">
+      <c r="H29" t="s" s="2">
         <v>321</v>
       </c>
-      <c r="I29" t="s" s="15">
+      <c r="I29" t="s" s="2">
         <v>322</v>
       </c>
-      <c r="J29" t="s" s="15">
+      <c r="J29" t="s" s="2">
         <v>323</v>
       </c>
-      <c r="K29" t="s" s="15">
+      <c r="K29" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L29" t="s" s="15">
+      <c r="L29" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M29" t="s" s="15">
+      <c r="M29" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N29" t="s" s="15">
+      <c r="N29" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O29" t="s" s="15">
+      <c r="O29" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="P29" t="s" s="15">
+      <c r="P29" t="s" s="2">
         <v>228</v>
       </c>
-      <c r="Q29" t="s" s="15">
+      <c r="Q29" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R29" t="s" s="15">
+      <c r="R29" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S29" t="s" s="15">
+      <c r="S29" t="s" s="2">
         <v>324</v>
       </c>
-      <c r="T29" s="11"/>
+      <c r="T29" s="3"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" t="s" s="15">
+      <c r="A30" t="s" s="2">
         <v>325</v>
       </c>
-      <c r="B30" t="s" s="15">
+      <c r="B30" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C30" t="s" s="15">
+      <c r="C30" t="s" s="2">
         <v>326</v>
       </c>
-      <c r="D30" t="s" s="15">
+      <c r="D30" t="s" s="2">
         <v>327</v>
       </c>
-      <c r="E30" t="s" s="15">
+      <c r="E30" t="s" s="2">
         <v>318</v>
       </c>
-      <c r="F30" t="s" s="15">
+      <c r="F30" t="s" s="2">
         <v>328</v>
       </c>
-      <c r="G30" t="s" s="15">
+      <c r="G30" t="s" s="2">
         <v>320</v>
       </c>
-      <c r="H30" t="s" s="15">
+      <c r="H30" t="s" s="2">
         <v>329</v>
       </c>
-      <c r="I30" t="s" s="15">
+      <c r="I30" t="s" s="2">
         <v>330</v>
       </c>
-      <c r="J30" t="s" s="15">
+      <c r="J30" t="s" s="2">
         <v>331</v>
       </c>
-      <c r="K30" t="s" s="15">
+      <c r="K30" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L30" t="s" s="15">
+      <c r="L30" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M30" t="s" s="15">
+      <c r="M30" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N30" t="s" s="15">
+      <c r="N30" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O30" t="s" s="15">
+      <c r="O30" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="P30" t="s" s="15">
+      <c r="P30" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="Q30" t="s" s="15">
+      <c r="Q30" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R30" t="s" s="15">
+      <c r="R30" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S30" t="s" s="15">
+      <c r="S30" t="s" s="2">
         <v>332</v>
       </c>
-      <c r="T30" s="11"/>
+      <c r="T30" s="3"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" t="s" s="15">
+      <c r="A31" t="s" s="2">
         <v>333</v>
       </c>
-      <c r="B31" t="s" s="15">
+      <c r="B31" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C31" t="s" s="15">
+      <c r="C31" t="s" s="2">
         <v>334</v>
       </c>
-      <c r="D31" t="s" s="15">
+      <c r="D31" t="s" s="2">
         <v>334</v>
       </c>
-      <c r="E31" t="s" s="15">
+      <c r="E31" t="s" s="2">
         <v>335</v>
       </c>
-      <c r="F31" t="s" s="15">
+      <c r="F31" t="s" s="2">
         <v>336</v>
       </c>
-      <c r="G31" t="s" s="15">
+      <c r="G31" t="s" s="2">
         <v>337</v>
       </c>
-      <c r="H31" t="s" s="15">
+      <c r="H31" t="s" s="2">
         <v>338</v>
       </c>
-      <c r="I31" t="s" s="15">
+      <c r="I31" t="s" s="2">
         <v>339</v>
       </c>
-      <c r="J31" t="s" s="15">
+      <c r="J31" t="s" s="2">
         <v>340</v>
       </c>
-      <c r="K31" t="s" s="15">
+      <c r="K31" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L31" t="s" s="15">
+      <c r="L31" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M31" t="s" s="15">
+      <c r="M31" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N31" t="s" s="15">
+      <c r="N31" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O31" t="s" s="15">
+      <c r="O31" t="s" s="2">
         <v>341</v>
       </c>
-      <c r="P31" t="s" s="15">
+      <c r="P31" t="s" s="2">
         <v>342</v>
       </c>
-      <c r="Q31" t="s" s="15">
+      <c r="Q31" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R31" t="s" s="15">
+      <c r="R31" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S31" s="16"/>
-      <c r="T31" s="11"/>
+      <c r="S31" s="3"/>
+      <c r="T31" s="3"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" t="s" s="15">
+      <c r="A32" t="s" s="2">
         <v>343</v>
       </c>
-      <c r="B32" t="s" s="15">
+      <c r="B32" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C32" t="s" s="15">
+      <c r="C32" t="s" s="2">
         <v>344</v>
       </c>
-      <c r="D32" t="s" s="15">
+      <c r="D32" t="s" s="2">
         <v>344</v>
       </c>
-      <c r="E32" t="s" s="15">
+      <c r="E32" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="F32" t="s" s="15">
+      <c r="F32" t="s" s="2">
         <v>346</v>
       </c>
-      <c r="G32" t="s" s="15">
+      <c r="G32" t="s" s="2">
         <v>347</v>
       </c>
-      <c r="H32" t="s" s="15">
+      <c r="H32" t="s" s="2">
         <v>348</v>
       </c>
-      <c r="I32" t="s" s="15">
+      <c r="I32" t="s" s="2">
         <v>349</v>
       </c>
-      <c r="J32" t="s" s="15">
+      <c r="J32" t="s" s="2">
         <v>350</v>
       </c>
-      <c r="K32" t="s" s="15">
+      <c r="K32" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L32" t="s" s="15">
+      <c r="L32" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M32" t="s" s="15">
+      <c r="M32" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N32" t="s" s="15">
+      <c r="N32" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O32" t="s" s="15">
+      <c r="O32" t="s" s="2">
         <v>314</v>
       </c>
-      <c r="P32" t="s" s="15">
+      <c r="P32" t="s" s="2">
         <v>351</v>
       </c>
-      <c r="Q32" t="s" s="15">
+      <c r="Q32" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R32" t="s" s="15">
+      <c r="R32" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S32" s="16"/>
-      <c r="T32" s="11"/>
+      <c r="S32" s="3"/>
+      <c r="T32" s="3"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" t="s" s="15">
+      <c r="A33" t="s" s="2">
         <v>352</v>
       </c>
-      <c r="B33" t="s" s="15">
+      <c r="B33" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C33" t="s" s="15">
+      <c r="C33" t="s" s="2">
         <v>353</v>
       </c>
-      <c r="D33" t="s" s="15">
+      <c r="D33" t="s" s="2">
         <v>353</v>
       </c>
-      <c r="E33" t="s" s="15">
+      <c r="E33" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F33" t="s" s="15">
+      <c r="F33" t="s" s="2">
         <v>354</v>
       </c>
-      <c r="G33" t="s" s="15">
+      <c r="G33" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H33" t="s" s="15">
+      <c r="H33" t="s" s="2">
         <v>355</v>
       </c>
-      <c r="I33" t="s" s="15">
+      <c r="I33" t="s" s="2">
         <v>356</v>
       </c>
-      <c r="J33" t="s" s="15">
+      <c r="J33" t="s" s="2">
         <v>357</v>
       </c>
-      <c r="K33" t="s" s="15">
+      <c r="K33" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L33" t="s" s="15">
+      <c r="L33" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M33" t="s" s="15">
+      <c r="M33" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N33" t="s" s="15">
+      <c r="N33" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O33" t="s" s="15">
+      <c r="O33" t="s" s="2">
         <v>358</v>
       </c>
-      <c r="P33" t="s" s="15">
+      <c r="P33" t="s" s="2">
         <v>359</v>
       </c>
-      <c r="Q33" t="s" s="15">
+      <c r="Q33" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R33" t="s" s="15">
+      <c r="R33" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S33" s="16"/>
-      <c r="T33" s="11"/>
+      <c r="S33" s="3"/>
+      <c r="T33" s="3"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" t="s" s="15">
+      <c r="A34" t="s" s="2">
         <v>360</v>
       </c>
-      <c r="B34" t="s" s="15">
+      <c r="B34" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C34" t="s" s="15">
+      <c r="C34" t="s" s="2">
         <v>361</v>
       </c>
-      <c r="D34" t="s" s="15">
+      <c r="D34" t="s" s="2">
         <v>361</v>
       </c>
-      <c r="E34" t="s" s="15">
+      <c r="E34" t="s" s="2">
         <v>335</v>
       </c>
-      <c r="F34" t="s" s="15">
+      <c r="F34" t="s" s="2">
         <v>362</v>
       </c>
-      <c r="G34" t="s" s="15">
+      <c r="G34" t="s" s="2">
         <v>337</v>
       </c>
-      <c r="H34" t="s" s="15">
+      <c r="H34" t="s" s="2">
         <v>363</v>
       </c>
-      <c r="I34" t="s" s="15">
+      <c r="I34" t="s" s="2">
         <v>364</v>
       </c>
-      <c r="J34" t="s" s="15">
+      <c r="J34" t="s" s="2">
         <v>365</v>
       </c>
-      <c r="K34" t="s" s="15">
+      <c r="K34" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L34" t="s" s="15">
+      <c r="L34" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M34" t="s" s="15">
+      <c r="M34" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N34" t="s" s="15">
+      <c r="N34" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O34" t="s" s="15">
+      <c r="O34" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="P34" t="s" s="15">
+      <c r="P34" t="s" s="2">
         <v>367</v>
       </c>
-      <c r="Q34" t="s" s="15">
+      <c r="Q34" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R34" t="s" s="15">
+      <c r="R34" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S34" s="16"/>
-      <c r="T34" s="11"/>
+      <c r="S34" s="3"/>
+      <c r="T34" s="3"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="A35" t="s" s="15">
+      <c r="A35" t="s" s="2">
         <v>368</v>
       </c>
-      <c r="B35" t="s" s="15">
+      <c r="B35" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C35" t="s" s="15">
+      <c r="C35" t="s" s="2">
         <v>369</v>
       </c>
-      <c r="D35" t="s" s="15">
+      <c r="D35" t="s" s="2">
         <v>369</v>
       </c>
-      <c r="E35" t="s" s="15">
+      <c r="E35" t="s" s="2">
         <v>370</v>
       </c>
-      <c r="F35" t="s" s="15">
+      <c r="F35" t="s" s="2">
         <v>371</v>
       </c>
-      <c r="G35" t="s" s="15">
+      <c r="G35" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="H35" t="s" s="15">
+      <c r="H35" t="s" s="2">
         <v>373</v>
       </c>
-      <c r="I35" t="s" s="15">
+      <c r="I35" t="s" s="2">
         <v>374</v>
       </c>
-      <c r="J35" t="s" s="15">
+      <c r="J35" t="s" s="2">
         <v>375</v>
       </c>
-      <c r="K35" t="s" s="15">
+      <c r="K35" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L35" t="s" s="15">
+      <c r="L35" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M35" t="s" s="15">
+      <c r="M35" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N35" t="s" s="15">
+      <c r="N35" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O35" t="s" s="15">
+      <c r="O35" t="s" s="2">
         <v>218</v>
       </c>
-      <c r="P35" t="s" s="15">
+      <c r="P35" t="s" s="2">
         <v>376</v>
       </c>
-      <c r="Q35" t="s" s="15">
+      <c r="Q35" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R35" t="s" s="15">
+      <c r="R35" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S35" s="16"/>
-      <c r="T35" s="11"/>
+      <c r="S35" s="3"/>
+      <c r="T35" s="3"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="A36" t="s" s="15">
+      <c r="A36" t="s" s="2">
         <v>377</v>
       </c>
-      <c r="B36" t="s" s="15">
+      <c r="B36" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C36" t="s" s="15">
+      <c r="C36" t="s" s="2">
         <v>378</v>
       </c>
-      <c r="D36" t="s" s="15">
+      <c r="D36" t="s" s="2">
         <v>378</v>
       </c>
-      <c r="E36" t="s" s="15">
+      <c r="E36" t="s" s="2">
         <v>279</v>
       </c>
-      <c r="F36" t="s" s="15">
+      <c r="F36" t="s" s="2">
         <v>379</v>
       </c>
-      <c r="G36" t="s" s="15">
+      <c r="G36" t="s" s="2">
         <v>281</v>
       </c>
-      <c r="H36" t="s" s="15">
+      <c r="H36" t="s" s="2">
         <v>380</v>
       </c>
-      <c r="I36" t="s" s="15">
+      <c r="I36" t="s" s="2">
         <v>381</v>
       </c>
-      <c r="J36" t="s" s="15">
+      <c r="J36" t="s" s="2">
         <v>382</v>
       </c>
-      <c r="K36" t="s" s="15">
+      <c r="K36" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L36" t="s" s="15">
+      <c r="L36" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M36" t="s" s="15">
+      <c r="M36" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N36" t="s" s="15">
+      <c r="N36" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O36" t="s" s="15">
+      <c r="O36" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="P36" s="17">
+      <c r="P36" s="5">
         <v>18.3333333333333</v>
       </c>
-      <c r="Q36" t="s" s="15">
+      <c r="Q36" t="s" s="2">
         <v>384</v>
       </c>
-      <c r="R36" t="s" s="15">
+      <c r="R36" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S36" t="s" s="15">
+      <c r="S36" t="s" s="2">
         <v>385</v>
       </c>
-      <c r="T36" s="11"/>
+      <c r="T36" s="3"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="A37" t="s" s="15">
+      <c r="A37" t="s" s="2">
         <v>386</v>
       </c>
-      <c r="B37" t="s" s="15">
+      <c r="B37" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C37" t="s" s="15">
+      <c r="C37" t="s" s="2">
         <v>387</v>
       </c>
-      <c r="D37" t="s" s="15">
+      <c r="D37" t="s" s="2">
         <v>387</v>
       </c>
-      <c r="E37" t="s" s="15">
+      <c r="E37" t="s" s="2">
         <v>388</v>
       </c>
-      <c r="F37" t="s" s="15">
+      <c r="F37" t="s" s="2">
         <v>389</v>
       </c>
-      <c r="G37" t="s" s="15">
+      <c r="G37" t="s" s="2">
         <v>390</v>
       </c>
-      <c r="H37" t="s" s="15">
+      <c r="H37" t="s" s="2">
         <v>391</v>
       </c>
-      <c r="I37" t="s" s="15">
+      <c r="I37" t="s" s="2">
         <v>392</v>
       </c>
-      <c r="J37" t="s" s="15">
+      <c r="J37" t="s" s="2">
         <v>393</v>
       </c>
-      <c r="K37" t="s" s="15">
+      <c r="K37" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L37" t="s" s="15">
+      <c r="L37" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M37" t="s" s="15">
+      <c r="M37" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N37" t="s" s="15">
+      <c r="N37" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O37" t="s" s="15">
+      <c r="O37" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="P37" t="s" s="15">
+      <c r="P37" t="s" s="2">
         <v>394</v>
       </c>
-      <c r="Q37" t="s" s="15">
+      <c r="Q37" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R37" t="s" s="15">
+      <c r="R37" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S37" s="16"/>
-      <c r="T37" s="11"/>
+      <c r="S37" s="3"/>
+      <c r="T37" s="3"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="A38" t="s" s="15">
+      <c r="A38" t="s" s="2">
         <v>395</v>
       </c>
-      <c r="B38" t="s" s="15">
+      <c r="B38" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" t="s" s="15">
+      <c r="C38" s="3"/>
+      <c r="D38" t="s" s="2">
         <v>396</v>
       </c>
-      <c r="E38" t="s" s="15">
+      <c r="E38" t="s" s="2">
         <v>397</v>
       </c>
-      <c r="F38" t="s" s="15">
+      <c r="F38" t="s" s="2">
         <v>398</v>
       </c>
-      <c r="G38" t="s" s="15">
+      <c r="G38" t="s" s="2">
         <v>399</v>
       </c>
-      <c r="H38" t="s" s="15">
+      <c r="H38" t="s" s="2">
         <v>400</v>
       </c>
-      <c r="I38" t="s" s="15">
+      <c r="I38" t="s" s="2">
         <v>401</v>
       </c>
-      <c r="J38" t="s" s="15">
+      <c r="J38" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="K38" t="s" s="15">
+      <c r="K38" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L38" t="s" s="15">
+      <c r="L38" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M38" t="s" s="15">
+      <c r="M38" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N38" t="s" s="15">
+      <c r="N38" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O38" t="s" s="15">
+      <c r="O38" t="s" s="2">
         <v>403</v>
       </c>
-      <c r="P38" t="s" s="15">
+      <c r="P38" t="s" s="2">
         <v>404</v>
       </c>
-      <c r="Q38" t="s" s="15">
+      <c r="Q38" t="s" s="2">
         <v>256</v>
       </c>
-      <c r="R38" t="s" s="15">
+      <c r="R38" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S38" t="s" s="15">
+      <c r="S38" t="s" s="2">
         <v>405</v>
       </c>
-      <c r="T38" s="11"/>
+      <c r="T38" s="3"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" t="s" s="15">
+      <c r="A39" t="s" s="2">
         <v>406</v>
       </c>
-      <c r="B39" t="s" s="15">
+      <c r="B39" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C39" t="s" s="15">
+      <c r="C39" t="s" s="2">
         <v>407</v>
       </c>
-      <c r="D39" t="s" s="15">
+      <c r="D39" t="s" s="2">
         <v>407</v>
       </c>
-      <c r="E39" t="s" s="15">
+      <c r="E39" t="s" s="2">
         <v>408</v>
       </c>
-      <c r="F39" t="s" s="15">
+      <c r="F39" t="s" s="2">
         <v>409</v>
       </c>
-      <c r="G39" t="s" s="15">
+      <c r="G39" t="s" s="2">
         <v>410</v>
       </c>
-      <c r="H39" t="s" s="15">
+      <c r="H39" t="s" s="2">
         <v>411</v>
       </c>
-      <c r="I39" t="s" s="15">
+      <c r="I39" t="s" s="2">
         <v>412</v>
       </c>
-      <c r="J39" t="s" s="15">
+      <c r="J39" t="s" s="2">
         <v>413</v>
       </c>
-      <c r="K39" t="s" s="15">
+      <c r="K39" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L39" t="s" s="15">
+      <c r="L39" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M39" t="s" s="15">
+      <c r="M39" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N39" t="s" s="15">
+      <c r="N39" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O39" t="s" s="15">
+      <c r="O39" t="s" s="2">
         <v>414</v>
       </c>
-      <c r="P39" t="s" s="15">
+      <c r="P39" t="s" s="2">
         <v>394</v>
       </c>
-      <c r="Q39" t="s" s="15">
+      <c r="Q39" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R39" t="s" s="15">
+      <c r="R39" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S39" s="16"/>
-      <c r="T39" s="11"/>
+      <c r="S39" s="3"/>
+      <c r="T39" s="3"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" t="s" s="15">
+      <c r="A40" t="s" s="2">
         <v>415</v>
       </c>
-      <c r="B40" t="s" s="15">
+      <c r="B40" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C40" t="s" s="15">
+      <c r="C40" t="s" s="2">
         <v>416</v>
       </c>
-      <c r="D40" t="s" s="15">
+      <c r="D40" t="s" s="2">
         <v>416</v>
       </c>
-      <c r="E40" t="s" s="15">
+      <c r="E40" t="s" s="2">
         <v>417</v>
       </c>
-      <c r="F40" t="s" s="15">
+      <c r="F40" t="s" s="2">
         <v>418</v>
       </c>
-      <c r="G40" t="s" s="15">
+      <c r="G40" t="s" s="2">
         <v>419</v>
       </c>
-      <c r="H40" t="s" s="15">
+      <c r="H40" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="I40" t="s" s="15">
+      <c r="I40" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="J40" t="s" s="15">
+      <c r="J40" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="K40" t="s" s="15">
+      <c r="K40" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L40" t="s" s="15">
+      <c r="L40" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M40" t="s" s="15">
+      <c r="M40" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N40" t="s" s="15">
+      <c r="N40" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O40" t="s" s="15">
+      <c r="O40" t="s" s="2">
         <v>296</v>
       </c>
-      <c r="P40" t="s" s="15">
+      <c r="P40" t="s" s="2">
         <v>423</v>
       </c>
-      <c r="Q40" t="s" s="15">
+      <c r="Q40" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R40" t="s" s="15">
+      <c r="R40" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S40" s="16"/>
-      <c r="T40" s="11"/>
+      <c r="S40" s="3"/>
+      <c r="T40" s="3"/>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" t="s" s="15">
+      <c r="A41" t="s" s="2">
         <v>424</v>
       </c>
-      <c r="B41" t="s" s="15">
+      <c r="B41" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C41" t="s" s="15">
+      <c r="C41" t="s" s="2">
         <v>425</v>
       </c>
-      <c r="D41" t="s" s="15">
+      <c r="D41" t="s" s="2">
         <v>425</v>
       </c>
-      <c r="E41" t="s" s="15">
+      <c r="E41" t="s" s="2">
         <v>426</v>
       </c>
-      <c r="F41" t="s" s="15">
+      <c r="F41" t="s" s="2">
         <v>427</v>
       </c>
-      <c r="G41" t="s" s="15">
+      <c r="G41" t="s" s="2">
         <v>428</v>
       </c>
-      <c r="H41" t="s" s="15">
+      <c r="H41" t="s" s="2">
         <v>429</v>
       </c>
-      <c r="I41" t="s" s="15">
+      <c r="I41" t="s" s="2">
         <v>430</v>
       </c>
-      <c r="J41" t="s" s="15">
+      <c r="J41" t="s" s="2">
         <v>431</v>
       </c>
-      <c r="K41" t="s" s="15">
+      <c r="K41" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L41" t="s" s="15">
+      <c r="L41" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M41" t="s" s="15">
+      <c r="M41" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N41" t="s" s="15">
+      <c r="N41" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O41" t="s" s="15">
+      <c r="O41" t="s" s="2">
         <v>432</v>
       </c>
-      <c r="P41" t="s" s="15">
+      <c r="P41" t="s" s="2">
         <v>433</v>
       </c>
-      <c r="Q41" t="s" s="15">
+      <c r="Q41" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R41" t="s" s="15">
+      <c r="R41" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S41" s="16"/>
-      <c r="T41" s="11"/>
+      <c r="S41" s="3"/>
+      <c r="T41" s="3"/>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" t="s" s="15">
+      <c r="A42" t="s" s="2">
         <v>434</v>
       </c>
-      <c r="B42" t="s" s="15">
+      <c r="B42" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C42" t="s" s="15">
+      <c r="C42" t="s" s="2">
         <v>435</v>
       </c>
-      <c r="D42" t="s" s="15">
+      <c r="D42" t="s" s="2">
         <v>435</v>
       </c>
-      <c r="E42" t="s" s="15">
+      <c r="E42" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="F42" t="s" s="15">
+      <c r="F42" t="s" s="2">
         <v>436</v>
       </c>
-      <c r="G42" t="s" s="15">
+      <c r="G42" t="s" s="2">
         <v>437</v>
       </c>
-      <c r="H42" t="s" s="15">
+      <c r="H42" t="s" s="2">
         <v>438</v>
       </c>
-      <c r="I42" t="s" s="15">
+      <c r="I42" t="s" s="2">
         <v>439</v>
       </c>
-      <c r="J42" t="s" s="15">
+      <c r="J42" t="s" s="2">
         <v>440</v>
       </c>
-      <c r="K42" t="s" s="15">
+      <c r="K42" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L42" t="s" s="15">
+      <c r="L42" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M42" t="s" s="15">
+      <c r="M42" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N42" t="s" s="15">
+      <c r="N42" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O42" t="s" s="15">
+      <c r="O42" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="P42" t="s" s="15">
+      <c r="P42" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="Q42" t="s" s="15">
+      <c r="Q42" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R42" t="s" s="15">
+      <c r="R42" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S42" s="16"/>
-      <c r="T42" s="11"/>
+      <c r="S42" s="3"/>
+      <c r="T42" s="3"/>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" t="s" s="15">
+      <c r="A43" t="s" s="2">
         <v>441</v>
       </c>
-      <c r="B43" t="s" s="15">
+      <c r="B43" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C43" t="s" s="15">
+      <c r="C43" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="D43" t="s" s="15">
+      <c r="D43" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="E43" t="s" s="15">
+      <c r="E43" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="F43" t="s" s="15">
+      <c r="F43" t="s" s="2">
         <v>443</v>
       </c>
-      <c r="G43" t="s" s="15">
+      <c r="G43" t="s" s="2">
         <v>444</v>
       </c>
-      <c r="H43" t="s" s="15">
+      <c r="H43" t="s" s="2">
         <v>445</v>
       </c>
-      <c r="I43" t="s" s="15">
+      <c r="I43" t="s" s="2">
         <v>446</v>
       </c>
-      <c r="J43" t="s" s="15">
+      <c r="J43" t="s" s="2">
         <v>447</v>
       </c>
-      <c r="K43" t="s" s="15">
+      <c r="K43" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L43" t="s" s="15">
+      <c r="L43" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M43" t="s" s="15">
+      <c r="M43" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N43" t="s" s="15">
+      <c r="N43" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O43" t="s" s="15">
+      <c r="O43" t="s" s="2">
         <v>448</v>
       </c>
-      <c r="P43" t="s" s="15">
+      <c r="P43" t="s" s="2">
         <v>449</v>
       </c>
-      <c r="Q43" t="s" s="15">
+      <c r="Q43" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R43" t="s" s="15">
+      <c r="R43" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S43" s="16"/>
-      <c r="T43" s="11"/>
+      <c r="S43" s="3"/>
+      <c r="T43" s="3"/>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="A44" t="s" s="15">
+      <c r="A44" t="s" s="2">
         <v>450</v>
       </c>
-      <c r="B44" t="s" s="15">
+      <c r="B44" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C44" t="s" s="15">
+      <c r="C44" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="D44" t="s" s="15">
+      <c r="D44" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="E44" t="s" s="15">
+      <c r="E44" t="s" s="2">
         <v>452</v>
       </c>
-      <c r="F44" t="s" s="15">
+      <c r="F44" t="s" s="2">
         <v>453</v>
       </c>
-      <c r="G44" t="s" s="15">
+      <c r="G44" t="s" s="2">
         <v>454</v>
       </c>
-      <c r="H44" t="s" s="15">
+      <c r="H44" t="s" s="2">
         <v>455</v>
       </c>
-      <c r="I44" t="s" s="15">
+      <c r="I44" t="s" s="2">
         <v>456</v>
       </c>
-      <c r="J44" t="s" s="15">
+      <c r="J44" t="s" s="2">
         <v>457</v>
       </c>
-      <c r="K44" t="s" s="15">
+      <c r="K44" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L44" t="s" s="15">
+      <c r="L44" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M44" t="s" s="15">
+      <c r="M44" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N44" t="s" s="15">
+      <c r="N44" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O44" t="s" s="15">
+      <c r="O44" t="s" s="2">
         <v>314</v>
       </c>
-      <c r="P44" t="s" s="15">
+      <c r="P44" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="Q44" t="s" s="15">
+      <c r="Q44" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R44" t="s" s="15">
+      <c r="R44" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S44" s="16"/>
-      <c r="T44" s="11"/>
+      <c r="S44" s="3"/>
+      <c r="T44" s="3"/>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="A45" t="s" s="15">
+      <c r="A45" t="s" s="2">
         <v>459</v>
       </c>
-      <c r="B45" t="s" s="15">
+      <c r="B45" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C45" t="s" s="15">
+      <c r="C45" t="s" s="2">
         <v>460</v>
       </c>
-      <c r="D45" t="s" s="15">
+      <c r="D45" t="s" s="2">
         <v>460</v>
       </c>
-      <c r="E45" t="s" s="15">
+      <c r="E45" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="F45" t="s" s="15">
+      <c r="F45" t="s" s="2">
         <v>461</v>
       </c>
-      <c r="G45" t="s" s="15">
+      <c r="G45" t="s" s="2">
         <v>347</v>
       </c>
-      <c r="H45" t="s" s="15">
+      <c r="H45" t="s" s="2">
         <v>462</v>
       </c>
-      <c r="I45" t="s" s="15">
+      <c r="I45" t="s" s="2">
         <v>463</v>
       </c>
-      <c r="J45" t="s" s="15">
+      <c r="J45" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="K45" t="s" s="15">
+      <c r="K45" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L45" t="s" s="15">
+      <c r="L45" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M45" t="s" s="15">
+      <c r="M45" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N45" t="s" s="15">
+      <c r="N45" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O45" t="s" s="15">
+      <c r="O45" t="s" s="2">
         <v>414</v>
       </c>
-      <c r="P45" t="s" s="15">
+      <c r="P45" t="s" s="2">
         <v>297</v>
       </c>
-      <c r="Q45" t="s" s="15">
+      <c r="Q45" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R45" t="s" s="15">
+      <c r="R45" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S45" s="16"/>
-      <c r="T45" s="11"/>
+      <c r="S45" s="3"/>
+      <c r="T45" s="3"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="A46" t="s" s="15">
+      <c r="A46" t="s" s="2">
         <v>465</v>
       </c>
-      <c r="B46" t="s" s="15">
+      <c r="B46" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C46" t="s" s="15">
+      <c r="C46" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="D46" t="s" s="15">
+      <c r="D46" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="E46" t="s" s="15">
+      <c r="E46" t="s" s="2">
         <v>467</v>
       </c>
-      <c r="F46" t="s" s="15">
+      <c r="F46" t="s" s="2">
         <v>468</v>
       </c>
-      <c r="G46" t="s" s="15">
+      <c r="G46" t="s" s="2">
         <v>469</v>
       </c>
-      <c r="H46" t="s" s="15">
+      <c r="H46" t="s" s="2">
         <v>470</v>
       </c>
-      <c r="I46" t="s" s="15">
+      <c r="I46" t="s" s="2">
         <v>471</v>
       </c>
-      <c r="J46" t="s" s="15">
+      <c r="J46" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="K46" t="s" s="15">
+      <c r="K46" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L46" t="s" s="15">
+      <c r="L46" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M46" t="s" s="15">
+      <c r="M46" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N46" t="s" s="15">
+      <c r="N46" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O46" t="s" s="15">
+      <c r="O46" t="s" s="2">
         <v>313</v>
       </c>
-      <c r="P46" t="s" s="15">
+      <c r="P46" t="s" s="2">
         <v>473</v>
       </c>
-      <c r="Q46" t="s" s="15">
+      <c r="Q46" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R46" t="s" s="15">
+      <c r="R46" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S46" s="16"/>
-      <c r="T46" s="11"/>
+      <c r="S46" s="3"/>
+      <c r="T46" s="3"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="A47" t="s" s="15">
+      <c r="A47" t="s" s="2">
         <v>474</v>
       </c>
-      <c r="B47" t="s" s="15">
+      <c r="B47" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C47" t="s" s="15">
+      <c r="C47" t="s" s="2">
         <v>475</v>
       </c>
-      <c r="D47" t="s" s="15">
+      <c r="D47" t="s" s="2">
         <v>475</v>
       </c>
-      <c r="E47" t="s" s="15">
+      <c r="E47" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="F47" t="s" s="15">
+      <c r="F47" t="s" s="2">
         <v>476</v>
       </c>
-      <c r="G47" t="s" s="15">
+      <c r="G47" t="s" s="2">
         <v>437</v>
       </c>
-      <c r="H47" t="s" s="15">
+      <c r="H47" t="s" s="2">
         <v>477</v>
       </c>
-      <c r="I47" t="s" s="15">
+      <c r="I47" t="s" s="2">
         <v>478</v>
       </c>
-      <c r="J47" t="s" s="15">
+      <c r="J47" t="s" s="2">
         <v>479</v>
       </c>
-      <c r="K47" t="s" s="15">
+      <c r="K47" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L47" t="s" s="15">
+      <c r="L47" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M47" t="s" s="15">
+      <c r="M47" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N47" t="s" s="15">
+      <c r="N47" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O47" t="s" s="15">
+      <c r="O47" t="s" s="2">
         <v>313</v>
       </c>
-      <c r="P47" t="s" s="15">
+      <c r="P47" t="s" s="2">
         <v>414</v>
       </c>
-      <c r="Q47" t="s" s="15">
+      <c r="Q47" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R47" t="s" s="15">
+      <c r="R47" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S47" s="16"/>
-      <c r="T47" s="11"/>
+      <c r="S47" s="3"/>
+      <c r="T47" s="3"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" t="s" s="15">
+      <c r="A48" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="B48" t="s" s="15">
+      <c r="B48" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C48" t="s" s="15">
+      <c r="C48" t="s" s="2">
         <v>481</v>
       </c>
-      <c r="D48" t="s" s="15">
+      <c r="D48" t="s" s="2">
         <v>481</v>
       </c>
-      <c r="E48" t="s" s="15">
+      <c r="E48" t="s" s="2">
         <v>250</v>
       </c>
-      <c r="F48" t="s" s="15">
+      <c r="F48" t="s" s="2">
         <v>482</v>
       </c>
-      <c r="G48" t="s" s="15">
+      <c r="G48" t="s" s="2">
         <v>483</v>
       </c>
-      <c r="H48" t="s" s="15">
+      <c r="H48" t="s" s="2">
         <v>484</v>
       </c>
-      <c r="I48" t="s" s="15">
+      <c r="I48" t="s" s="2">
         <v>485</v>
       </c>
-      <c r="J48" t="s" s="15">
+      <c r="J48" t="s" s="2">
         <v>486</v>
       </c>
-      <c r="K48" t="s" s="15">
+      <c r="K48" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L48" t="s" s="15">
+      <c r="L48" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M48" t="s" s="15">
+      <c r="M48" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N48" t="s" s="15">
+      <c r="N48" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O48" t="s" s="15">
+      <c r="O48" t="s" s="2">
         <v>449</v>
       </c>
-      <c r="P48" t="s" s="15">
+      <c r="P48" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="Q48" t="s" s="15">
+      <c r="Q48" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R48" t="s" s="15">
+      <c r="R48" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S48" s="16"/>
-      <c r="T48" s="11"/>
+      <c r="S48" s="3"/>
+      <c r="T48" s="3"/>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" t="s" s="15">
+      <c r="A49" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="B49" t="s" s="15">
+      <c r="B49" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C49" t="s" s="15">
+      <c r="C49" t="s" s="2">
         <v>488</v>
       </c>
-      <c r="D49" t="s" s="15">
+      <c r="D49" t="s" s="2">
         <v>488</v>
       </c>
-      <c r="E49" t="s" s="15">
+      <c r="E49" t="s" s="2">
         <v>489</v>
       </c>
-      <c r="F49" t="s" s="15">
+      <c r="F49" t="s" s="2">
         <v>490</v>
       </c>
-      <c r="G49" t="s" s="15">
+      <c r="G49" t="s" s="2">
         <v>491</v>
       </c>
-      <c r="H49" t="s" s="15">
+      <c r="H49" t="s" s="2">
         <v>492</v>
       </c>
-      <c r="I49" t="s" s="15">
+      <c r="I49" t="s" s="2">
         <v>493</v>
       </c>
-      <c r="J49" t="s" s="15">
+      <c r="J49" t="s" s="2">
         <v>494</v>
       </c>
-      <c r="K49" t="s" s="15">
+      <c r="K49" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L49" t="s" s="15">
+      <c r="L49" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M49" t="s" s="15">
+      <c r="M49" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N49" t="s" s="15">
+      <c r="N49" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O49" t="s" s="15">
+      <c r="O49" t="s" s="2">
         <v>495</v>
       </c>
-      <c r="P49" t="s" s="15">
+      <c r="P49" t="s" s="2">
         <v>496</v>
       </c>
-      <c r="Q49" t="s" s="15">
+      <c r="Q49" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R49" t="s" s="15">
+      <c r="R49" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S49" s="16"/>
-      <c r="T49" s="11"/>
+      <c r="S49" s="3"/>
+      <c r="T49" s="3"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="A50" t="s" s="15">
+      <c r="A50" t="s" s="2">
         <v>497</v>
       </c>
-      <c r="B50" t="s" s="15">
+      <c r="B50" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C50" t="s" s="15">
+      <c r="C50" t="s" s="2">
         <v>498</v>
       </c>
-      <c r="D50" t="s" s="15">
+      <c r="D50" t="s" s="2">
         <v>498</v>
       </c>
-      <c r="E50" t="s" s="15">
+      <c r="E50" t="s" s="2">
         <v>499</v>
       </c>
-      <c r="F50" t="s" s="15">
+      <c r="F50" t="s" s="2">
         <v>500</v>
       </c>
-      <c r="G50" t="s" s="15">
+      <c r="G50" t="s" s="2">
         <v>501</v>
       </c>
-      <c r="H50" t="s" s="15">
+      <c r="H50" t="s" s="2">
         <v>502</v>
       </c>
-      <c r="I50" t="s" s="15">
+      <c r="I50" t="s" s="2">
         <v>503</v>
       </c>
-      <c r="J50" t="s" s="15">
+      <c r="J50" t="s" s="2">
         <v>504</v>
       </c>
-      <c r="K50" t="s" s="15">
+      <c r="K50" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L50" t="s" s="15">
+      <c r="L50" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M50" t="s" s="15">
+      <c r="M50" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N50" t="s" s="15">
+      <c r="N50" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O50" t="s" s="15">
+      <c r="O50" t="s" s="2">
         <v>505</v>
       </c>
-      <c r="P50" t="s" s="15">
+      <c r="P50" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="Q50" t="s" s="15">
+      <c r="Q50" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R50" t="s" s="15">
+      <c r="R50" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S50" s="16"/>
-      <c r="T50" s="11"/>
+      <c r="S50" s="3"/>
+      <c r="T50" s="3"/>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="A51" s="18"/>
-      <c r="B51" s="18"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18"/>
-      <c r="F51" s="18"/>
-      <c r="G51" s="18"/>
-      <c r="H51" s="18"/>
-      <c r="I51" s="18"/>
-      <c r="J51" s="18"/>
-      <c r="K51" s="18"/>
-      <c r="L51" s="18"/>
-      <c r="M51" s="18"/>
-      <c r="N51" s="18"/>
-      <c r="O51" s="18"/>
-      <c r="P51" s="18"/>
-      <c r="Q51" s="18"/>
-      <c r="R51" s="18"/>
-      <c r="S51" s="18"/>
-      <c r="T51" s="4"/>
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
+      <c r="O51" s="3"/>
+      <c r="P51" s="3"/>
+      <c r="Q51" s="3"/>
+      <c r="R51" s="3"/>
+      <c r="S51" s="3"/>
+      <c r="T51" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add prediction workflow, AusRAP comparison and delivery documentation (#8)
* Update prediction workflow and add evaluation/ausrap modules

* feat: add AusRAP references to prediction exports

* fix: align imagery concurrency defaults and tests

* fix: align batch inputs and location eligibility

* feat: add iRAP comparison evaluation and evidence

* feat: add reproducible offline prediction example

* docs: standardize documentation and folder guides

* chore: untrack building caches and remove notebook credentials
</commit_message>
<xml_diff>
--- a/data/templates/model_dataset_template.xlsx
+++ b/data/templates/model_dataset_template.xlsx
@@ -1540,7 +1540,7 @@
     <numFmt numFmtId="0" formatCode="General"/>
     <numFmt numFmtId="59" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -1556,39 +1556,16 @@
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="16"/>
-      <color indexed="8"/>
-      <name val="Aptos"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Aptos"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Aptos"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="9"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1598,76 +1575,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="10"/>
+        <color indexed="9"/>
       </left>
       <right style="thin">
-        <color indexed="10"/>
+        <color indexed="9"/>
       </right>
       <top style="thin">
-        <color indexed="10"/>
+        <color indexed="9"/>
       </top>
       <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
+        <color indexed="9"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1677,62 +1594,23 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="59" fontId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -1752,8 +1630,7 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="ffa5a5a5"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1952,7 +1829,7 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="19050" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
@@ -1989,10 +1866,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -2231,7 +2108,7 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="19050" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
@@ -2540,10 +2417,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -2786,7 +2663,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E35"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="27" style="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="1" customWidth="1"/>
@@ -2803,445 +2680,445 @@
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="4"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" t="s" s="6">
+      <c r="A3" t="s" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="4"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" t="s" s="8">
+      <c r="A4" t="s" s="2">
         <v>2</v>
       </c>
-      <c r="B4" t="s" s="9">
+      <c r="B4" t="s" s="2">
         <v>3</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="11"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" t="s" s="8">
+      <c r="A5" t="s" s="2">
         <v>4</v>
       </c>
-      <c r="B5" t="s" s="9">
+      <c r="B5" t="s" s="2">
         <v>5</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="11"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" t="s" s="8">
+      <c r="A6" t="s" s="2">
         <v>6</v>
       </c>
-      <c r="B6" t="s" s="9">
+      <c r="B6" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="11"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" t="s" s="8">
+      <c r="A7" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="B7" t="s" s="9">
+      <c r="B7" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="11"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" t="s" s="8">
+      <c r="A8" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="B8" t="s" s="9">
+      <c r="B8" t="s" s="2">
         <v>11</v>
       </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="11"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" t="s" s="8">
+      <c r="A9" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="B9" t="s" s="9">
+      <c r="B9" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="11"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
     </row>
     <row r="10" ht="26.35" customHeight="1">
-      <c r="A10" t="s" s="8">
+      <c r="A10" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="B10" t="s" s="9">
+      <c r="B10" t="s" s="2">
         <v>15</v>
       </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="11"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
     </row>
     <row r="11" ht="26.35" customHeight="1">
-      <c r="A11" t="s" s="8">
+      <c r="A11" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="B11" t="s" s="9">
+      <c r="B11" t="s" s="2">
         <v>17</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="11"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" t="s" s="8">
+      <c r="A12" t="s" s="2">
         <v>18</v>
       </c>
-      <c r="B12" t="s" s="9">
+      <c r="B12" t="s" s="2">
         <v>19</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="11"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="4"/>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="4"/>
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" t="s" s="6">
+      <c r="A15" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="4"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" t="s" s="8">
+      <c r="A16" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="B16" t="s" s="8">
+      <c r="B16" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="C16" t="s" s="8">
+      <c r="C16" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="D16" t="s" s="8">
+      <c r="D16" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="E16" s="11"/>
+      <c r="E16" s="3"/>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" t="s" s="9">
+      <c r="A17" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B17" t="s" s="9">
+      <c r="B17" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C17" t="s" s="9">
+      <c r="C17" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D17" t="s" s="9">
+      <c r="D17" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="E17" s="11"/>
+      <c r="E17" s="3"/>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" t="s" s="9">
+      <c r="A18" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="B18" t="s" s="9">
+      <c r="B18" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C18" t="s" s="9">
+      <c r="C18" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D18" t="s" s="9">
+      <c r="D18" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="E18" s="11"/>
+      <c r="E18" s="3"/>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" t="s" s="9">
+      <c r="A19" t="s" s="2">
         <v>30</v>
       </c>
-      <c r="B19" t="s" s="9">
+      <c r="B19" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C19" t="s" s="9">
+      <c r="C19" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D19" t="s" s="9">
+      <c r="D19" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="E19" s="11"/>
+      <c r="E19" s="3"/>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" t="s" s="9">
+      <c r="A20" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="B20" t="s" s="9">
+      <c r="B20" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C20" t="s" s="9">
+      <c r="C20" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D20" t="s" s="9">
+      <c r="D20" t="s" s="2">
         <v>34</v>
       </c>
-      <c r="E20" s="11"/>
+      <c r="E20" s="3"/>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" t="s" s="9">
+      <c r="A21" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="B21" t="s" s="9">
+      <c r="B21" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C21" t="s" s="9">
+      <c r="C21" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D21" t="s" s="9">
+      <c r="D21" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="E21" s="11"/>
+      <c r="E21" s="3"/>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" t="s" s="9">
+      <c r="A22" t="s" s="2">
         <v>37</v>
       </c>
-      <c r="B22" t="s" s="9">
+      <c r="B22" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C22" t="s" s="9">
+      <c r="C22" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D22" t="s" s="9">
+      <c r="D22" t="s" s="2">
         <v>39</v>
       </c>
-      <c r="E22" s="11"/>
+      <c r="E22" s="3"/>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" t="s" s="9">
+      <c r="A23" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="B23" t="s" s="9">
+      <c r="B23" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C23" t="s" s="9">
+      <c r="C23" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D23" t="s" s="9">
+      <c r="D23" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="E23" s="11"/>
+      <c r="E23" s="3"/>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" t="s" s="9">
+      <c r="A24" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="B24" t="s" s="9">
+      <c r="B24" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C24" t="s" s="9">
+      <c r="C24" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D24" t="s" s="9">
+      <c r="D24" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="E24" s="11"/>
+      <c r="E24" s="3"/>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="A25" t="s" s="9">
+      <c r="A25" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="B25" t="s" s="9">
+      <c r="B25" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C25" t="s" s="9">
+      <c r="C25" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D25" t="s" s="9">
+      <c r="D25" t="s" s="2">
         <v>45</v>
       </c>
-      <c r="E25" s="11"/>
+      <c r="E25" s="3"/>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" t="s" s="9">
+      <c r="A26" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="B26" t="s" s="9">
+      <c r="B26" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C26" t="s" s="9">
+      <c r="C26" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D26" t="s" s="9">
+      <c r="D26" t="s" s="2">
         <v>47</v>
       </c>
-      <c r="E26" s="11"/>
+      <c r="E26" s="3"/>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="A27" t="s" s="9">
+      <c r="A27" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B27" t="s" s="9">
+      <c r="B27" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C27" t="s" s="9">
+      <c r="C27" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D27" t="s" s="9">
+      <c r="D27" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="E27" s="11"/>
+      <c r="E27" s="3"/>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="A28" t="s" s="9">
+      <c r="A28" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="B28" t="s" s="9">
+      <c r="B28" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C28" t="s" s="9">
+      <c r="C28" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D28" t="s" s="9">
+      <c r="D28" t="s" s="2">
         <v>51</v>
       </c>
-      <c r="E28" s="11"/>
+      <c r="E28" s="3"/>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="A29" t="s" s="9">
+      <c r="A29" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="B29" t="s" s="9">
+      <c r="B29" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="C29" t="s" s="9">
+      <c r="C29" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D29" t="s" s="9">
+      <c r="D29" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="E29" s="11"/>
+      <c r="E29" s="3"/>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="A30" t="s" s="9">
+      <c r="A30" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="B30" t="s" s="9">
+      <c r="B30" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="C30" t="s" s="9">
+      <c r="C30" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D30" t="s" s="9">
+      <c r="D30" t="s" s="2">
         <v>56</v>
       </c>
-      <c r="E30" s="11"/>
+      <c r="E30" s="3"/>
     </row>
     <row r="31" ht="15" customHeight="1">
-      <c r="A31" t="s" s="9">
+      <c r="A31" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="B31" t="s" s="9">
+      <c r="B31" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C31" t="s" s="9">
+      <c r="C31" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D31" t="s" s="9">
+      <c r="D31" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="E31" s="11"/>
+      <c r="E31" s="3"/>
     </row>
     <row r="32" ht="15" customHeight="1">
-      <c r="A32" t="s" s="9">
+      <c r="A32" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="B32" t="s" s="9">
+      <c r="B32" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C32" t="s" s="9">
+      <c r="C32" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D32" t="s" s="9">
+      <c r="D32" t="s" s="2">
         <v>60</v>
       </c>
-      <c r="E32" s="11"/>
+      <c r="E32" s="3"/>
     </row>
     <row r="33" ht="15" customHeight="1">
-      <c r="A33" t="s" s="9">
+      <c r="A33" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B33" t="s" s="9">
+      <c r="B33" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C33" t="s" s="9">
+      <c r="C33" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D33" t="s" s="9">
+      <c r="D33" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="E33" s="11"/>
+      <c r="E33" s="3"/>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" t="s" s="9">
+      <c r="A34" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="B34" t="s" s="9">
+      <c r="B34" t="s" s="2">
         <v>64</v>
       </c>
-      <c r="C34" t="s" s="9">
+      <c r="C34" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D34" t="s" s="9">
+      <c r="D34" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="E34" s="11"/>
+      <c r="E34" s="3"/>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="A35" t="s" s="9">
+      <c r="A35" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="B35" t="s" s="9">
+      <c r="B35" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C35" t="s" s="9">
+      <c r="C35" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D35" t="s" s="9">
+      <c r="D35" t="s" s="2">
         <v>67</v>
       </c>
-      <c r="E35" s="11"/>
+      <c r="E35" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -3269,2957 +3146,2957 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:T51"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="16" style="13" customWidth="1"/>
-    <col min="2" max="2" width="14" style="13" customWidth="1"/>
-    <col min="3" max="4" width="18" style="13" customWidth="1"/>
-    <col min="5" max="6" width="12" style="13" customWidth="1"/>
-    <col min="7" max="7" width="24" style="13" customWidth="1"/>
-    <col min="8" max="8" width="34" style="13" customWidth="1"/>
-    <col min="9" max="11" width="14" style="13" customWidth="1"/>
-    <col min="12" max="12" width="34" style="13" customWidth="1"/>
-    <col min="13" max="13" width="15" style="13" customWidth="1"/>
-    <col min="14" max="14" width="14" style="13" customWidth="1"/>
-    <col min="15" max="16" width="20" style="13" customWidth="1"/>
-    <col min="17" max="17" width="24" style="13" customWidth="1"/>
-    <col min="18" max="18" width="18" style="13" customWidth="1"/>
-    <col min="19" max="19" width="50" style="13" customWidth="1"/>
-    <col min="20" max="20" width="8.85156" style="13" customWidth="1"/>
-    <col min="21" max="16384" width="8.85156" style="13" customWidth="1"/>
+    <col min="1" max="1" width="16" style="4" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
+    <col min="3" max="4" width="18" style="4" customWidth="1"/>
+    <col min="5" max="6" width="12" style="4" customWidth="1"/>
+    <col min="7" max="7" width="24" style="4" customWidth="1"/>
+    <col min="8" max="8" width="34" style="4" customWidth="1"/>
+    <col min="9" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="34" style="4" customWidth="1"/>
+    <col min="13" max="13" width="15" style="4" customWidth="1"/>
+    <col min="14" max="14" width="14" style="4" customWidth="1"/>
+    <col min="15" max="16" width="20" style="4" customWidth="1"/>
+    <col min="17" max="17" width="24" style="4" customWidth="1"/>
+    <col min="18" max="18" width="18" style="4" customWidth="1"/>
+    <col min="19" max="19" width="50" style="4" customWidth="1"/>
+    <col min="20" max="20" width="8.85156" style="4" customWidth="1"/>
+    <col min="21" max="16384" width="8.85156" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" t="s" s="14">
+      <c r="A1" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B1" t="s" s="14">
+      <c r="B1" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="C1" t="s" s="14">
+      <c r="C1" t="s" s="2">
         <v>30</v>
       </c>
-      <c r="D1" t="s" s="14">
+      <c r="D1" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="E1" t="s" s="14">
+      <c r="E1" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="F1" t="s" s="14">
+      <c r="F1" t="s" s="2">
         <v>37</v>
       </c>
-      <c r="G1" t="s" s="14">
+      <c r="G1" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="H1" t="s" s="14">
+      <c r="H1" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="I1" t="s" s="14">
+      <c r="I1" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="J1" t="s" s="14">
+      <c r="J1" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="K1" t="s" s="14">
+      <c r="K1" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="L1" t="s" s="14">
+      <c r="L1" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="M1" t="s" s="14">
+      <c r="M1" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="N1" t="s" s="14">
+      <c r="N1" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="O1" t="s" s="14">
+      <c r="O1" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="P1" t="s" s="14">
+      <c r="P1" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="Q1" t="s" s="14">
+      <c r="Q1" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="R1" t="s" s="14">
+      <c r="R1" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="S1" t="s" s="14">
+      <c r="S1" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="T1" s="11"/>
+      <c r="T1" s="3"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" t="s" s="15">
+      <c r="A2" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B2" t="s" s="15">
+      <c r="B2" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C2" t="s" s="15">
+      <c r="C2" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="D2" t="s" s="15">
+      <c r="D2" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="E2" t="s" s="15">
+      <c r="E2" t="s" s="2">
         <v>71</v>
       </c>
-      <c r="F2" t="s" s="15">
+      <c r="F2" t="s" s="2">
         <v>72</v>
       </c>
-      <c r="G2" t="s" s="15">
+      <c r="G2" t="s" s="2">
         <v>73</v>
       </c>
-      <c r="H2" t="s" s="15">
+      <c r="H2" t="s" s="2">
         <v>74</v>
       </c>
-      <c r="I2" t="s" s="15">
+      <c r="I2" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="J2" t="s" s="15">
+      <c r="J2" t="s" s="2">
         <v>76</v>
       </c>
-      <c r="K2" t="s" s="15">
+      <c r="K2" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L2" t="s" s="15">
+      <c r="L2" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M2" t="s" s="15">
+      <c r="M2" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N2" t="s" s="15">
+      <c r="N2" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O2" t="s" s="15">
+      <c r="O2" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="P2" t="s" s="15">
+      <c r="P2" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="Q2" t="s" s="15">
+      <c r="Q2" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R2" t="s" s="15">
+      <c r="R2" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S2" s="16"/>
-      <c r="T2" s="11"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" t="s" s="15">
+      <c r="A3" t="s" s="2">
         <v>85</v>
       </c>
-      <c r="B3" t="s" s="15">
+      <c r="B3" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C3" t="s" s="15">
+      <c r="C3" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="D3" t="s" s="15">
+      <c r="D3" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="E3" t="s" s="15">
+      <c r="E3" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F3" t="s" s="15">
+      <c r="F3" t="s" s="2">
         <v>88</v>
       </c>
-      <c r="G3" t="s" s="15">
+      <c r="G3" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H3" t="s" s="15">
+      <c r="H3" t="s" s="2">
         <v>90</v>
       </c>
-      <c r="I3" t="s" s="15">
+      <c r="I3" t="s" s="2">
         <v>91</v>
       </c>
-      <c r="J3" t="s" s="15">
+      <c r="J3" t="s" s="2">
         <v>92</v>
       </c>
-      <c r="K3" t="s" s="15">
+      <c r="K3" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L3" t="s" s="15">
+      <c r="L3" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M3" t="s" s="15">
+      <c r="M3" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N3" t="s" s="15">
+      <c r="N3" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O3" t="s" s="15">
+      <c r="O3" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="P3" t="s" s="15">
+      <c r="P3" t="s" s="2">
         <v>95</v>
       </c>
-      <c r="Q3" t="s" s="15">
+      <c r="Q3" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R3" t="s" s="15">
+      <c r="R3" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S3" s="16"/>
-      <c r="T3" s="11"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" t="s" s="15">
+      <c r="A4" t="s" s="2">
         <v>96</v>
       </c>
-      <c r="B4" t="s" s="15">
+      <c r="B4" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C4" t="s" s="15">
+      <c r="C4" t="s" s="2">
         <v>97</v>
       </c>
-      <c r="D4" t="s" s="15">
+      <c r="D4" t="s" s="2">
         <v>97</v>
       </c>
-      <c r="E4" t="s" s="15">
+      <c r="E4" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="F4" t="s" s="15">
+      <c r="F4" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="G4" t="s" s="15">
+      <c r="G4" t="s" s="2">
         <v>100</v>
       </c>
-      <c r="H4" t="s" s="15">
+      <c r="H4" t="s" s="2">
         <v>101</v>
       </c>
-      <c r="I4" t="s" s="15">
+      <c r="I4" t="s" s="2">
         <v>102</v>
       </c>
-      <c r="J4" t="s" s="15">
+      <c r="J4" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="K4" t="s" s="15">
+      <c r="K4" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L4" t="s" s="15">
+      <c r="L4" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M4" t="s" s="15">
+      <c r="M4" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N4" t="s" s="15">
+      <c r="N4" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O4" t="s" s="15">
+      <c r="O4" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="P4" t="s" s="15">
+      <c r="P4" t="s" s="2">
         <v>105</v>
       </c>
-      <c r="Q4" t="s" s="15">
+      <c r="Q4" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R4" t="s" s="15">
+      <c r="R4" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S4" s="16"/>
-      <c r="T4" s="11"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" t="s" s="15">
+      <c r="A5" t="s" s="2">
         <v>106</v>
       </c>
-      <c r="B5" t="s" s="15">
+      <c r="B5" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C5" t="s" s="15">
+      <c r="C5" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="D5" t="s" s="15">
+      <c r="D5" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="E5" t="s" s="15">
+      <c r="E5" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F5" t="s" s="15">
+      <c r="F5" t="s" s="2">
         <v>108</v>
       </c>
-      <c r="G5" t="s" s="15">
+      <c r="G5" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H5" t="s" s="15">
+      <c r="H5" t="s" s="2">
         <v>109</v>
       </c>
-      <c r="I5" t="s" s="15">
+      <c r="I5" t="s" s="2">
         <v>110</v>
       </c>
-      <c r="J5" t="s" s="15">
+      <c r="J5" t="s" s="2">
         <v>111</v>
       </c>
-      <c r="K5" t="s" s="15">
+      <c r="K5" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L5" t="s" s="15">
+      <c r="L5" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M5" t="s" s="15">
+      <c r="M5" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N5" t="s" s="15">
+      <c r="N5" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O5" t="s" s="15">
+      <c r="O5" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="P5" t="s" s="15">
+      <c r="P5" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="Q5" t="s" s="15">
+      <c r="Q5" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R5" t="s" s="15">
+      <c r="R5" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S5" s="16"/>
-      <c r="T5" s="11"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" t="s" s="15">
+      <c r="A6" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="B6" t="s" s="15">
+      <c r="B6" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C6" t="s" s="15">
+      <c r="C6" t="s" s="2">
         <v>115</v>
       </c>
-      <c r="D6" t="s" s="15">
+      <c r="D6" t="s" s="2">
         <v>115</v>
       </c>
-      <c r="E6" t="s" s="15">
+      <c r="E6" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F6" t="s" s="15">
+      <c r="F6" t="s" s="2">
         <v>116</v>
       </c>
-      <c r="G6" t="s" s="15">
+      <c r="G6" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H6" t="s" s="15">
+      <c r="H6" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="I6" t="s" s="15">
+      <c r="I6" t="s" s="2">
         <v>118</v>
       </c>
-      <c r="J6" t="s" s="15">
+      <c r="J6" t="s" s="2">
         <v>119</v>
       </c>
-      <c r="K6" t="s" s="15">
+      <c r="K6" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L6" t="s" s="15">
+      <c r="L6" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M6" t="s" s="15">
+      <c r="M6" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N6" t="s" s="15">
+      <c r="N6" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O6" t="s" s="15">
+      <c r="O6" t="s" s="2">
         <v>120</v>
       </c>
-      <c r="P6" t="s" s="15">
+      <c r="P6" t="s" s="2">
         <v>121</v>
       </c>
-      <c r="Q6" t="s" s="15">
+      <c r="Q6" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R6" t="s" s="15">
+      <c r="R6" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S6" s="16"/>
-      <c r="T6" s="11"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" t="s" s="15">
+      <c r="A7" t="s" s="2">
         <v>122</v>
       </c>
-      <c r="B7" t="s" s="15">
+      <c r="B7" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C7" t="s" s="15">
+      <c r="C7" t="s" s="2">
         <v>123</v>
       </c>
-      <c r="D7" t="s" s="15">
+      <c r="D7" t="s" s="2">
         <v>123</v>
       </c>
-      <c r="E7" t="s" s="15">
+      <c r="E7" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F7" t="s" s="15">
+      <c r="F7" t="s" s="2">
         <v>124</v>
       </c>
-      <c r="G7" t="s" s="15">
+      <c r="G7" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H7" t="s" s="15">
+      <c r="H7" t="s" s="2">
         <v>125</v>
       </c>
-      <c r="I7" t="s" s="15">
+      <c r="I7" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="J7" t="s" s="15">
+      <c r="J7" t="s" s="2">
         <v>127</v>
       </c>
-      <c r="K7" t="s" s="15">
+      <c r="K7" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L7" t="s" s="15">
+      <c r="L7" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M7" t="s" s="15">
+      <c r="M7" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N7" t="s" s="15">
+      <c r="N7" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O7" t="s" s="15">
+      <c r="O7" t="s" s="2">
         <v>128</v>
       </c>
-      <c r="P7" t="s" s="15">
+      <c r="P7" t="s" s="2">
         <v>129</v>
       </c>
-      <c r="Q7" t="s" s="15">
+      <c r="Q7" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R7" t="s" s="15">
+      <c r="R7" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S7" s="16"/>
-      <c r="T7" s="11"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" t="s" s="15">
+      <c r="A8" t="s" s="2">
         <v>130</v>
       </c>
-      <c r="B8" t="s" s="15">
+      <c r="B8" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C8" t="s" s="15">
+      <c r="C8" t="s" s="2">
         <v>131</v>
       </c>
-      <c r="D8" t="s" s="15">
+      <c r="D8" t="s" s="2">
         <v>131</v>
       </c>
-      <c r="E8" t="s" s="15">
+      <c r="E8" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F8" t="s" s="15">
+      <c r="F8" t="s" s="2">
         <v>132</v>
       </c>
-      <c r="G8" t="s" s="15">
+      <c r="G8" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H8" t="s" s="15">
+      <c r="H8" t="s" s="2">
         <v>133</v>
       </c>
-      <c r="I8" t="s" s="15">
+      <c r="I8" t="s" s="2">
         <v>134</v>
       </c>
-      <c r="J8" t="s" s="15">
+      <c r="J8" t="s" s="2">
         <v>135</v>
       </c>
-      <c r="K8" t="s" s="15">
+      <c r="K8" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L8" t="s" s="15">
+      <c r="L8" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M8" t="s" s="15">
+      <c r="M8" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N8" t="s" s="15">
+      <c r="N8" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O8" t="s" s="15">
+      <c r="O8" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="P8" t="s" s="15">
+      <c r="P8" t="s" s="2">
         <v>137</v>
       </c>
-      <c r="Q8" t="s" s="15">
+      <c r="Q8" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R8" t="s" s="15">
+      <c r="R8" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S8" s="16"/>
-      <c r="T8" s="11"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" t="s" s="15">
+      <c r="A9" t="s" s="2">
         <v>138</v>
       </c>
-      <c r="B9" t="s" s="15">
+      <c r="B9" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C9" t="s" s="15">
+      <c r="C9" t="s" s="2">
         <v>139</v>
       </c>
-      <c r="D9" t="s" s="15">
+      <c r="D9" t="s" s="2">
         <v>139</v>
       </c>
-      <c r="E9" t="s" s="15">
+      <c r="E9" t="s" s="2">
         <v>140</v>
       </c>
-      <c r="F9" t="s" s="15">
+      <c r="F9" t="s" s="2">
         <v>141</v>
       </c>
-      <c r="G9" t="s" s="15">
+      <c r="G9" t="s" s="2">
         <v>142</v>
       </c>
-      <c r="H9" t="s" s="15">
+      <c r="H9" t="s" s="2">
         <v>143</v>
       </c>
-      <c r="I9" t="s" s="15">
+      <c r="I9" t="s" s="2">
         <v>144</v>
       </c>
-      <c r="J9" t="s" s="15">
+      <c r="J9" t="s" s="2">
         <v>145</v>
       </c>
-      <c r="K9" t="s" s="15">
+      <c r="K9" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L9" t="s" s="15">
+      <c r="L9" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M9" t="s" s="15">
+      <c r="M9" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N9" t="s" s="15">
+      <c r="N9" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O9" t="s" s="15">
+      <c r="O9" t="s" s="2">
         <v>146</v>
       </c>
-      <c r="P9" t="s" s="15">
+      <c r="P9" t="s" s="2">
         <v>147</v>
       </c>
-      <c r="Q9" t="s" s="15">
+      <c r="Q9" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R9" t="s" s="15">
+      <c r="R9" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S9" s="16"/>
-      <c r="T9" s="11"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" t="s" s="15">
+      <c r="A10" t="s" s="2">
         <v>148</v>
       </c>
-      <c r="B10" t="s" s="15">
+      <c r="B10" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C10" t="s" s="15">
+      <c r="C10" t="s" s="2">
         <v>149</v>
       </c>
-      <c r="D10" t="s" s="15">
+      <c r="D10" t="s" s="2">
         <v>149</v>
       </c>
-      <c r="E10" t="s" s="15">
+      <c r="E10" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F10" t="s" s="15">
+      <c r="F10" t="s" s="2">
         <v>150</v>
       </c>
-      <c r="G10" t="s" s="15">
+      <c r="G10" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H10" t="s" s="15">
+      <c r="H10" t="s" s="2">
         <v>151</v>
       </c>
-      <c r="I10" t="s" s="15">
+      <c r="I10" t="s" s="2">
         <v>152</v>
       </c>
-      <c r="J10" t="s" s="15">
+      <c r="J10" t="s" s="2">
         <v>153</v>
       </c>
-      <c r="K10" t="s" s="15">
+      <c r="K10" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L10" t="s" s="15">
+      <c r="L10" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M10" t="s" s="15">
+      <c r="M10" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N10" t="s" s="15">
+      <c r="N10" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O10" t="s" s="15">
+      <c r="O10" t="s" s="2">
         <v>154</v>
       </c>
-      <c r="P10" t="s" s="15">
+      <c r="P10" t="s" s="2">
         <v>155</v>
       </c>
-      <c r="Q10" t="s" s="15">
+      <c r="Q10" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R10" t="s" s="15">
+      <c r="R10" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S10" s="16"/>
-      <c r="T10" s="11"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" t="s" s="15">
+      <c r="A11" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="B11" t="s" s="15">
+      <c r="B11" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C11" t="s" s="15">
+      <c r="C11" t="s" s="2">
         <v>157</v>
       </c>
-      <c r="D11" t="s" s="15">
+      <c r="D11" t="s" s="2">
         <v>157</v>
       </c>
-      <c r="E11" t="s" s="15">
+      <c r="E11" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F11" t="s" s="15">
+      <c r="F11" t="s" s="2">
         <v>158</v>
       </c>
-      <c r="G11" t="s" s="15">
+      <c r="G11" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H11" t="s" s="15">
+      <c r="H11" t="s" s="2">
         <v>159</v>
       </c>
-      <c r="I11" t="s" s="15">
+      <c r="I11" t="s" s="2">
         <v>160</v>
       </c>
-      <c r="J11" t="s" s="15">
+      <c r="J11" t="s" s="2">
         <v>161</v>
       </c>
-      <c r="K11" t="s" s="15">
+      <c r="K11" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L11" t="s" s="15">
+      <c r="L11" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M11" t="s" s="15">
+      <c r="M11" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N11" t="s" s="15">
+      <c r="N11" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O11" t="s" s="15">
+      <c r="O11" t="s" s="2">
         <v>162</v>
       </c>
-      <c r="P11" t="s" s="15">
+      <c r="P11" t="s" s="2">
         <v>163</v>
       </c>
-      <c r="Q11" t="s" s="15">
+      <c r="Q11" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R11" t="s" s="15">
+      <c r="R11" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S11" s="16"/>
-      <c r="T11" s="11"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" t="s" s="15">
+      <c r="A12" t="s" s="2">
         <v>164</v>
       </c>
-      <c r="B12" t="s" s="15">
+      <c r="B12" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C12" t="s" s="15">
+      <c r="C12" t="s" s="2">
         <v>165</v>
       </c>
-      <c r="D12" t="s" s="15">
+      <c r="D12" t="s" s="2">
         <v>165</v>
       </c>
-      <c r="E12" t="s" s="15">
+      <c r="E12" t="s" s="2">
         <v>166</v>
       </c>
-      <c r="F12" t="s" s="15">
+      <c r="F12" t="s" s="2">
         <v>167</v>
       </c>
-      <c r="G12" t="s" s="15">
+      <c r="G12" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="H12" t="s" s="15">
+      <c r="H12" t="s" s="2">
         <v>169</v>
       </c>
-      <c r="I12" t="s" s="15">
+      <c r="I12" t="s" s="2">
         <v>170</v>
       </c>
-      <c r="J12" t="s" s="15">
+      <c r="J12" t="s" s="2">
         <v>171</v>
       </c>
-      <c r="K12" t="s" s="15">
+      <c r="K12" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L12" t="s" s="15">
+      <c r="L12" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M12" t="s" s="15">
+      <c r="M12" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N12" t="s" s="15">
+      <c r="N12" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O12" t="s" s="15">
+      <c r="O12" t="s" s="2">
         <v>172</v>
       </c>
-      <c r="P12" t="s" s="15">
+      <c r="P12" t="s" s="2">
         <v>173</v>
       </c>
-      <c r="Q12" t="s" s="15">
+      <c r="Q12" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R12" t="s" s="15">
+      <c r="R12" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S12" s="16"/>
-      <c r="T12" s="11"/>
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" t="s" s="15">
+      <c r="A13" t="s" s="2">
         <v>174</v>
       </c>
-      <c r="B13" t="s" s="15">
+      <c r="B13" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C13" t="s" s="15">
+      <c r="C13" t="s" s="2">
         <v>175</v>
       </c>
-      <c r="D13" t="s" s="15">
+      <c r="D13" t="s" s="2">
         <v>175</v>
       </c>
-      <c r="E13" t="s" s="15">
+      <c r="E13" t="s" s="2">
         <v>166</v>
       </c>
-      <c r="F13" t="s" s="15">
+      <c r="F13" t="s" s="2">
         <v>176</v>
       </c>
-      <c r="G13" t="s" s="15">
+      <c r="G13" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="H13" t="s" s="15">
+      <c r="H13" t="s" s="2">
         <v>177</v>
       </c>
-      <c r="I13" t="s" s="15">
+      <c r="I13" t="s" s="2">
         <v>178</v>
       </c>
-      <c r="J13" t="s" s="15">
+      <c r="J13" t="s" s="2">
         <v>179</v>
       </c>
-      <c r="K13" t="s" s="15">
+      <c r="K13" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L13" t="s" s="15">
+      <c r="L13" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M13" t="s" s="15">
+      <c r="M13" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N13" t="s" s="15">
+      <c r="N13" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O13" t="s" s="15">
+      <c r="O13" t="s" s="2">
         <v>128</v>
       </c>
-      <c r="P13" t="s" s="15">
+      <c r="P13" t="s" s="2">
         <v>180</v>
       </c>
-      <c r="Q13" t="s" s="15">
+      <c r="Q13" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R13" t="s" s="15">
+      <c r="R13" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S13" s="16"/>
-      <c r="T13" s="11"/>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" t="s" s="15">
+      <c r="A14" t="s" s="2">
         <v>181</v>
       </c>
-      <c r="B14" t="s" s="15">
+      <c r="B14" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C14" t="s" s="15">
+      <c r="C14" t="s" s="2">
         <v>182</v>
       </c>
-      <c r="D14" t="s" s="15">
+      <c r="D14" t="s" s="2">
         <v>182</v>
       </c>
-      <c r="E14" t="s" s="15">
+      <c r="E14" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F14" t="s" s="15">
+      <c r="F14" t="s" s="2">
         <v>183</v>
       </c>
-      <c r="G14" t="s" s="15">
+      <c r="G14" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H14" t="s" s="15">
+      <c r="H14" t="s" s="2">
         <v>184</v>
       </c>
-      <c r="I14" t="s" s="15">
+      <c r="I14" t="s" s="2">
         <v>185</v>
       </c>
-      <c r="J14" t="s" s="15">
+      <c r="J14" t="s" s="2">
         <v>186</v>
       </c>
-      <c r="K14" t="s" s="15">
+      <c r="K14" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L14" t="s" s="15">
+      <c r="L14" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M14" t="s" s="15">
+      <c r="M14" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N14" t="s" s="15">
+      <c r="N14" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O14" t="s" s="15">
+      <c r="O14" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="P14" t="s" s="15">
+      <c r="P14" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="Q14" t="s" s="15">
+      <c r="Q14" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R14" t="s" s="15">
+      <c r="R14" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S14" s="16"/>
-      <c r="T14" s="11"/>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" t="s" s="15">
+      <c r="A15" t="s" s="2">
         <v>187</v>
       </c>
-      <c r="B15" t="s" s="15">
+      <c r="B15" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C15" t="s" s="15">
+      <c r="C15" t="s" s="2">
         <v>188</v>
       </c>
-      <c r="D15" t="s" s="15">
+      <c r="D15" t="s" s="2">
         <v>188</v>
       </c>
-      <c r="E15" t="s" s="15">
+      <c r="E15" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F15" t="s" s="15">
+      <c r="F15" t="s" s="2">
         <v>189</v>
       </c>
-      <c r="G15" t="s" s="15">
+      <c r="G15" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H15" t="s" s="15">
+      <c r="H15" t="s" s="2">
         <v>190</v>
       </c>
-      <c r="I15" t="s" s="15">
+      <c r="I15" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="J15" t="s" s="15">
+      <c r="J15" t="s" s="2">
         <v>192</v>
       </c>
-      <c r="K15" t="s" s="15">
+      <c r="K15" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L15" t="s" s="15">
+      <c r="L15" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M15" t="s" s="15">
+      <c r="M15" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N15" t="s" s="15">
+      <c r="N15" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O15" t="s" s="15">
+      <c r="O15" t="s" s="2">
         <v>193</v>
       </c>
-      <c r="P15" t="s" s="15">
+      <c r="P15" t="s" s="2">
         <v>194</v>
       </c>
-      <c r="Q15" t="s" s="15">
+      <c r="Q15" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R15" t="s" s="15">
+      <c r="R15" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S15" s="16"/>
-      <c r="T15" s="11"/>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" t="s" s="15">
+      <c r="A16" t="s" s="2">
         <v>195</v>
       </c>
-      <c r="B16" t="s" s="15">
+      <c r="B16" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C16" t="s" s="15">
+      <c r="C16" t="s" s="2">
         <v>196</v>
       </c>
-      <c r="D16" t="s" s="15">
+      <c r="D16" t="s" s="2">
         <v>196</v>
       </c>
-      <c r="E16" t="s" s="15">
+      <c r="E16" t="s" s="2">
         <v>71</v>
       </c>
-      <c r="F16" t="s" s="15">
+      <c r="F16" t="s" s="2">
         <v>197</v>
       </c>
-      <c r="G16" t="s" s="15">
+      <c r="G16" t="s" s="2">
         <v>198</v>
       </c>
-      <c r="H16" t="s" s="15">
+      <c r="H16" t="s" s="2">
         <v>199</v>
       </c>
-      <c r="I16" t="s" s="15">
+      <c r="I16" t="s" s="2">
         <v>200</v>
       </c>
-      <c r="J16" t="s" s="15">
+      <c r="J16" t="s" s="2">
         <v>201</v>
       </c>
-      <c r="K16" t="s" s="15">
+      <c r="K16" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L16" t="s" s="15">
+      <c r="L16" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M16" t="s" s="15">
+      <c r="M16" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N16" t="s" s="15">
+      <c r="N16" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O16" t="s" s="15">
+      <c r="O16" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="P16" t="s" s="15">
+      <c r="P16" t="s" s="2">
         <v>202</v>
       </c>
-      <c r="Q16" t="s" s="15">
+      <c r="Q16" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R16" t="s" s="15">
+      <c r="R16" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S16" s="16"/>
-      <c r="T16" s="11"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" t="s" s="15">
+      <c r="A17" t="s" s="2">
         <v>203</v>
       </c>
-      <c r="B17" t="s" s="15">
+      <c r="B17" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C17" t="s" s="15">
+      <c r="C17" t="s" s="2">
         <v>204</v>
       </c>
-      <c r="D17" t="s" s="15">
+      <c r="D17" t="s" s="2">
         <v>204</v>
       </c>
-      <c r="E17" t="s" s="15">
+      <c r="E17" t="s" s="2">
         <v>205</v>
       </c>
-      <c r="F17" t="s" s="15">
+      <c r="F17" t="s" s="2">
         <v>206</v>
       </c>
-      <c r="G17" t="s" s="15">
+      <c r="G17" t="s" s="2">
         <v>207</v>
       </c>
-      <c r="H17" t="s" s="15">
+      <c r="H17" t="s" s="2">
         <v>208</v>
       </c>
-      <c r="I17" t="s" s="15">
+      <c r="I17" t="s" s="2">
         <v>209</v>
       </c>
-      <c r="J17" t="s" s="15">
+      <c r="J17" t="s" s="2">
         <v>210</v>
       </c>
-      <c r="K17" t="s" s="15">
+      <c r="K17" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L17" t="s" s="15">
+      <c r="L17" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M17" t="s" s="15">
+      <c r="M17" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N17" t="s" s="15">
+      <c r="N17" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O17" t="s" s="15">
+      <c r="O17" t="s" s="2">
         <v>211</v>
       </c>
-      <c r="P17" t="s" s="15">
+      <c r="P17" t="s" s="2">
         <v>194</v>
       </c>
-      <c r="Q17" t="s" s="15">
+      <c r="Q17" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R17" t="s" s="15">
+      <c r="R17" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S17" s="16"/>
-      <c r="T17" s="11"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" t="s" s="15">
+      <c r="A18" t="s" s="2">
         <v>212</v>
       </c>
-      <c r="B18" t="s" s="15">
+      <c r="B18" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C18" t="s" s="15">
+      <c r="C18" t="s" s="2">
         <v>213</v>
       </c>
-      <c r="D18" t="s" s="15">
+      <c r="D18" t="s" s="2">
         <v>213</v>
       </c>
-      <c r="E18" t="s" s="15">
+      <c r="E18" t="s" s="2">
         <v>166</v>
       </c>
-      <c r="F18" t="s" s="15">
+      <c r="F18" t="s" s="2">
         <v>214</v>
       </c>
-      <c r="G18" t="s" s="15">
+      <c r="G18" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="H18" t="s" s="15">
+      <c r="H18" t="s" s="2">
         <v>215</v>
       </c>
-      <c r="I18" t="s" s="15">
+      <c r="I18" t="s" s="2">
         <v>216</v>
       </c>
-      <c r="J18" t="s" s="15">
+      <c r="J18" t="s" s="2">
         <v>217</v>
       </c>
-      <c r="K18" t="s" s="15">
+      <c r="K18" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L18" t="s" s="15">
+      <c r="L18" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M18" t="s" s="15">
+      <c r="M18" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N18" t="s" s="15">
+      <c r="N18" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O18" t="s" s="15">
+      <c r="O18" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="P18" t="s" s="15">
+      <c r="P18" t="s" s="2">
         <v>218</v>
       </c>
-      <c r="Q18" t="s" s="15">
+      <c r="Q18" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R18" t="s" s="15">
+      <c r="R18" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S18" s="16"/>
-      <c r="T18" s="11"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" t="s" s="15">
+      <c r="A19" t="s" s="2">
         <v>219</v>
       </c>
-      <c r="B19" t="s" s="15">
+      <c r="B19" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C19" t="s" s="15">
+      <c r="C19" t="s" s="2">
         <v>221</v>
       </c>
-      <c r="D19" t="s" s="15">
+      <c r="D19" t="s" s="2">
         <v>221</v>
       </c>
-      <c r="E19" t="s" s="15">
+      <c r="E19" t="s" s="2">
         <v>222</v>
       </c>
-      <c r="F19" t="s" s="15">
+      <c r="F19" t="s" s="2">
         <v>223</v>
       </c>
-      <c r="G19" t="s" s="15">
+      <c r="G19" t="s" s="2">
         <v>224</v>
       </c>
-      <c r="H19" t="s" s="15">
+      <c r="H19" t="s" s="2">
         <v>225</v>
       </c>
-      <c r="I19" t="s" s="15">
+      <c r="I19" t="s" s="2">
         <v>226</v>
       </c>
-      <c r="J19" t="s" s="15">
+      <c r="J19" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="K19" t="s" s="15">
+      <c r="K19" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L19" t="s" s="15">
+      <c r="L19" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M19" t="s" s="15">
+      <c r="M19" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N19" t="s" s="15">
+      <c r="N19" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O19" t="s" s="15">
+      <c r="O19" t="s" s="2">
         <v>228</v>
       </c>
-      <c r="P19" t="s" s="15">
+      <c r="P19" t="s" s="2">
         <v>229</v>
       </c>
-      <c r="Q19" t="s" s="15">
+      <c r="Q19" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R19" t="s" s="15">
+      <c r="R19" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S19" s="16"/>
-      <c r="T19" s="11"/>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" t="s" s="15">
+      <c r="A20" t="s" s="2">
         <v>230</v>
       </c>
-      <c r="B20" t="s" s="15">
+      <c r="B20" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C20" t="s" s="15">
+      <c r="C20" t="s" s="2">
         <v>231</v>
       </c>
-      <c r="D20" t="s" s="15">
+      <c r="D20" t="s" s="2">
         <v>231</v>
       </c>
-      <c r="E20" t="s" s="15">
+      <c r="E20" t="s" s="2">
         <v>232</v>
       </c>
-      <c r="F20" t="s" s="15">
+      <c r="F20" t="s" s="2">
         <v>233</v>
       </c>
-      <c r="G20" t="s" s="15">
+      <c r="G20" t="s" s="2">
         <v>234</v>
       </c>
-      <c r="H20" t="s" s="15">
+      <c r="H20" t="s" s="2">
         <v>235</v>
       </c>
-      <c r="I20" t="s" s="15">
+      <c r="I20" t="s" s="2">
         <v>236</v>
       </c>
-      <c r="J20" t="s" s="15">
+      <c r="J20" t="s" s="2">
         <v>237</v>
       </c>
-      <c r="K20" t="s" s="15">
+      <c r="K20" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L20" t="s" s="15">
+      <c r="L20" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M20" t="s" s="15">
+      <c r="M20" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N20" t="s" s="15">
+      <c r="N20" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O20" t="s" s="15">
+      <c r="O20" t="s" s="2">
         <v>238</v>
       </c>
-      <c r="P20" t="s" s="15">
+      <c r="P20" t="s" s="2">
         <v>218</v>
       </c>
-      <c r="Q20" t="s" s="15">
+      <c r="Q20" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R20" t="s" s="15">
+      <c r="R20" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S20" s="16"/>
-      <c r="T20" s="11"/>
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" t="s" s="15">
+      <c r="A21" t="s" s="2">
         <v>239</v>
       </c>
-      <c r="B21" t="s" s="15">
+      <c r="B21" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C21" t="s" s="15">
+      <c r="C21" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="D21" t="s" s="15">
+      <c r="D21" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="E21" t="s" s="15">
+      <c r="E21" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="F21" t="s" s="15">
+      <c r="F21" t="s" s="2">
         <v>242</v>
       </c>
-      <c r="G21" t="s" s="15">
+      <c r="G21" t="s" s="2">
         <v>243</v>
       </c>
-      <c r="H21" t="s" s="15">
+      <c r="H21" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="I21" t="s" s="15">
+      <c r="I21" t="s" s="2">
         <v>245</v>
       </c>
-      <c r="J21" t="s" s="15">
+      <c r="J21" t="s" s="2">
         <v>246</v>
       </c>
-      <c r="K21" t="s" s="15">
+      <c r="K21" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L21" t="s" s="15">
+      <c r="L21" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M21" t="s" s="15">
+      <c r="M21" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N21" t="s" s="15">
+      <c r="N21" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O21" t="s" s="15">
+      <c r="O21" t="s" s="2">
         <v>202</v>
       </c>
-      <c r="P21" t="s" s="15">
+      <c r="P21" t="s" s="2">
         <v>247</v>
       </c>
-      <c r="Q21" t="s" s="15">
+      <c r="Q21" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R21" t="s" s="15">
+      <c r="R21" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S21" s="16"/>
-      <c r="T21" s="11"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" t="s" s="15">
+      <c r="A22" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="B22" t="s" s="15">
+      <c r="B22" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C22" t="s" s="15">
+      <c r="C22" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="D22" t="s" s="15">
+      <c r="D22" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="E22" t="s" s="15">
+      <c r="E22" t="s" s="2">
         <v>250</v>
       </c>
-      <c r="F22" t="s" s="15">
+      <c r="F22" t="s" s="2">
         <v>251</v>
       </c>
-      <c r="G22" t="s" s="15">
+      <c r="G22" t="s" s="2">
         <v>252</v>
       </c>
-      <c r="H22" t="s" s="15">
+      <c r="H22" t="s" s="2">
         <v>253</v>
       </c>
-      <c r="I22" t="s" s="15">
+      <c r="I22" t="s" s="2">
         <v>254</v>
       </c>
-      <c r="J22" t="s" s="15">
+      <c r="J22" t="s" s="2">
         <v>255</v>
       </c>
-      <c r="K22" t="s" s="15">
+      <c r="K22" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L22" t="s" s="15">
+      <c r="L22" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M22" t="s" s="15">
+      <c r="M22" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N22" t="s" s="15">
+      <c r="N22" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O22" s="17">
+      <c r="O22" s="5">
         <v>87</v>
       </c>
-      <c r="P22" s="17">
+      <c r="P22" s="5">
         <v>17.3333333333333</v>
       </c>
-      <c r="Q22" t="s" s="15">
+      <c r="Q22" t="s" s="2">
         <v>256</v>
       </c>
-      <c r="R22" t="s" s="15">
+      <c r="R22" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S22" t="s" s="15">
+      <c r="S22" t="s" s="2">
         <v>257</v>
       </c>
-      <c r="T22" s="11"/>
+      <c r="T22" s="3"/>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" t="s" s="15">
+      <c r="A23" t="s" s="2">
         <v>258</v>
       </c>
-      <c r="B23" t="s" s="15">
+      <c r="B23" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C23" t="s" s="15">
+      <c r="C23" t="s" s="2">
         <v>259</v>
       </c>
-      <c r="D23" t="s" s="15">
+      <c r="D23" t="s" s="2">
         <v>259</v>
       </c>
-      <c r="E23" t="s" s="15">
+      <c r="E23" t="s" s="2">
         <v>260</v>
       </c>
-      <c r="F23" t="s" s="15">
+      <c r="F23" t="s" s="2">
         <v>261</v>
       </c>
-      <c r="G23" t="s" s="15">
+      <c r="G23" t="s" s="2">
         <v>262</v>
       </c>
-      <c r="H23" t="s" s="15">
+      <c r="H23" t="s" s="2">
         <v>263</v>
       </c>
-      <c r="I23" t="s" s="15">
+      <c r="I23" t="s" s="2">
         <v>264</v>
       </c>
-      <c r="J23" t="s" s="15">
+      <c r="J23" t="s" s="2">
         <v>265</v>
       </c>
-      <c r="K23" t="s" s="15">
+      <c r="K23" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L23" t="s" s="15">
+      <c r="L23" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M23" t="s" s="15">
+      <c r="M23" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N23" t="s" s="15">
+      <c r="N23" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O23" t="s" s="15">
+      <c r="O23" t="s" s="2">
         <v>266</v>
       </c>
-      <c r="P23" t="s" s="15">
+      <c r="P23" t="s" s="2">
         <v>266</v>
       </c>
-      <c r="Q23" t="s" s="15">
+      <c r="Q23" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R23" t="s" s="15">
+      <c r="R23" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S23" s="16"/>
-      <c r="T23" s="11"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" t="s" s="15">
+      <c r="A24" t="s" s="2">
         <v>267</v>
       </c>
-      <c r="B24" t="s" s="15">
+      <c r="B24" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C24" t="s" s="15">
+      <c r="C24" t="s" s="2">
         <v>268</v>
       </c>
-      <c r="D24" t="s" s="15">
+      <c r="D24" t="s" s="2">
         <v>268</v>
       </c>
-      <c r="E24" t="s" s="15">
+      <c r="E24" t="s" s="2">
         <v>269</v>
       </c>
-      <c r="F24" t="s" s="15">
+      <c r="F24" t="s" s="2">
         <v>270</v>
       </c>
-      <c r="G24" t="s" s="15">
+      <c r="G24" t="s" s="2">
         <v>271</v>
       </c>
-      <c r="H24" t="s" s="15">
+      <c r="H24" t="s" s="2">
         <v>272</v>
       </c>
-      <c r="I24" t="s" s="15">
+      <c r="I24" t="s" s="2">
         <v>273</v>
       </c>
-      <c r="J24" t="s" s="15">
+      <c r="J24" t="s" s="2">
         <v>274</v>
       </c>
-      <c r="K24" t="s" s="15">
+      <c r="K24" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L24" t="s" s="15">
+      <c r="L24" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M24" t="s" s="15">
+      <c r="M24" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N24" t="s" s="15">
+      <c r="N24" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O24" t="s" s="15">
+      <c r="O24" t="s" s="2">
         <v>275</v>
       </c>
-      <c r="P24" t="s" s="15">
+      <c r="P24" t="s" s="2">
         <v>276</v>
       </c>
-      <c r="Q24" t="s" s="15">
+      <c r="Q24" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R24" t="s" s="15">
+      <c r="R24" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S24" s="16"/>
-      <c r="T24" s="11"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" t="s" s="15">
+      <c r="A25" t="s" s="2">
         <v>277</v>
       </c>
-      <c r="B25" t="s" s="15">
+      <c r="B25" t="s" s="2">
         <v>220</v>
       </c>
-      <c r="C25" t="s" s="15">
+      <c r="C25" t="s" s="2">
         <v>278</v>
       </c>
-      <c r="D25" t="s" s="15">
+      <c r="D25" t="s" s="2">
         <v>278</v>
       </c>
-      <c r="E25" t="s" s="15">
+      <c r="E25" t="s" s="2">
         <v>279</v>
       </c>
-      <c r="F25" t="s" s="15">
+      <c r="F25" t="s" s="2">
         <v>280</v>
       </c>
-      <c r="G25" t="s" s="15">
+      <c r="G25" t="s" s="2">
         <v>281</v>
       </c>
-      <c r="H25" t="s" s="15">
+      <c r="H25" t="s" s="2">
         <v>282</v>
       </c>
-      <c r="I25" t="s" s="15">
+      <c r="I25" t="s" s="2">
         <v>283</v>
       </c>
-      <c r="J25" t="s" s="15">
+      <c r="J25" t="s" s="2">
         <v>284</v>
       </c>
-      <c r="K25" t="s" s="15">
+      <c r="K25" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L25" t="s" s="15">
+      <c r="L25" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M25" t="s" s="15">
+      <c r="M25" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N25" t="s" s="15">
+      <c r="N25" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O25" t="s" s="15">
+      <c r="O25" t="s" s="2">
         <v>285</v>
       </c>
-      <c r="P25" t="s" s="15">
+      <c r="P25" t="s" s="2">
         <v>286</v>
       </c>
-      <c r="Q25" t="s" s="15">
+      <c r="Q25" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R25" t="s" s="15">
+      <c r="R25" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S25" s="16"/>
-      <c r="T25" s="11"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" t="s" s="15">
+      <c r="A26" t="s" s="2">
         <v>287</v>
       </c>
-      <c r="B26" t="s" s="15">
+      <c r="B26" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C26" t="s" s="15">
+      <c r="C26" t="s" s="2">
         <v>289</v>
       </c>
-      <c r="D26" t="s" s="15">
+      <c r="D26" t="s" s="2">
         <v>289</v>
       </c>
-      <c r="E26" t="s" s="15">
+      <c r="E26" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="F26" t="s" s="15">
+      <c r="F26" t="s" s="2">
         <v>291</v>
       </c>
-      <c r="G26" t="s" s="15">
+      <c r="G26" t="s" s="2">
         <v>292</v>
       </c>
-      <c r="H26" t="s" s="15">
+      <c r="H26" t="s" s="2">
         <v>293</v>
       </c>
-      <c r="I26" t="s" s="15">
+      <c r="I26" t="s" s="2">
         <v>294</v>
       </c>
-      <c r="J26" t="s" s="15">
+      <c r="J26" t="s" s="2">
         <v>295</v>
       </c>
-      <c r="K26" t="s" s="15">
+      <c r="K26" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L26" t="s" s="15">
+      <c r="L26" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M26" t="s" s="15">
+      <c r="M26" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N26" t="s" s="15">
+      <c r="N26" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O26" t="s" s="15">
+      <c r="O26" t="s" s="2">
         <v>296</v>
       </c>
-      <c r="P26" t="s" s="15">
+      <c r="P26" t="s" s="2">
         <v>297</v>
       </c>
-      <c r="Q26" t="s" s="15">
+      <c r="Q26" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R26" t="s" s="15">
+      <c r="R26" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S26" s="16"/>
-      <c r="T26" s="11"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" t="s" s="15">
+      <c r="A27" t="s" s="2">
         <v>298</v>
       </c>
-      <c r="B27" t="s" s="15">
+      <c r="B27" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C27" t="s" s="15">
+      <c r="C27" t="s" s="2">
         <v>299</v>
       </c>
-      <c r="D27" t="s" s="15">
+      <c r="D27" t="s" s="2">
         <v>299</v>
       </c>
-      <c r="E27" t="s" s="15">
+      <c r="E27" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="F27" t="s" s="15">
+      <c r="F27" t="s" s="2">
         <v>300</v>
       </c>
-      <c r="G27" t="s" s="15">
+      <c r="G27" t="s" s="2">
         <v>292</v>
       </c>
-      <c r="H27" t="s" s="15">
+      <c r="H27" t="s" s="2">
         <v>301</v>
       </c>
-      <c r="I27" t="s" s="15">
+      <c r="I27" t="s" s="2">
         <v>302</v>
       </c>
-      <c r="J27" t="s" s="15">
+      <c r="J27" t="s" s="2">
         <v>303</v>
       </c>
-      <c r="K27" t="s" s="15">
+      <c r="K27" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L27" t="s" s="15">
+      <c r="L27" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M27" t="s" s="15">
+      <c r="M27" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N27" t="s" s="15">
+      <c r="N27" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O27" t="s" s="15">
+      <c r="O27" t="s" s="2">
         <v>304</v>
       </c>
-      <c r="P27" t="s" s="15">
+      <c r="P27" t="s" s="2">
         <v>238</v>
       </c>
-      <c r="Q27" t="s" s="15">
+      <c r="Q27" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R27" t="s" s="15">
+      <c r="R27" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S27" s="16"/>
-      <c r="T27" s="11"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" t="s" s="15">
+      <c r="A28" t="s" s="2">
         <v>305</v>
       </c>
-      <c r="B28" t="s" s="15">
+      <c r="B28" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C28" t="s" s="15">
+      <c r="C28" t="s" s="2">
         <v>306</v>
       </c>
-      <c r="D28" t="s" s="15">
+      <c r="D28" t="s" s="2">
         <v>306</v>
       </c>
-      <c r="E28" t="s" s="15">
+      <c r="E28" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="F28" t="s" s="15">
+      <c r="F28" t="s" s="2">
         <v>308</v>
       </c>
-      <c r="G28" t="s" s="15">
+      <c r="G28" t="s" s="2">
         <v>309</v>
       </c>
-      <c r="H28" t="s" s="15">
+      <c r="H28" t="s" s="2">
         <v>310</v>
       </c>
-      <c r="I28" t="s" s="15">
+      <c r="I28" t="s" s="2">
         <v>311</v>
       </c>
-      <c r="J28" t="s" s="15">
+      <c r="J28" t="s" s="2">
         <v>312</v>
       </c>
-      <c r="K28" t="s" s="15">
+      <c r="K28" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L28" t="s" s="15">
+      <c r="L28" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M28" t="s" s="15">
+      <c r="M28" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N28" t="s" s="15">
+      <c r="N28" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O28" t="s" s="15">
+      <c r="O28" t="s" s="2">
         <v>313</v>
       </c>
-      <c r="P28" t="s" s="15">
+      <c r="P28" t="s" s="2">
         <v>314</v>
       </c>
-      <c r="Q28" t="s" s="15">
+      <c r="Q28" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R28" t="s" s="15">
+      <c r="R28" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S28" s="16"/>
-      <c r="T28" s="11"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" t="s" s="15">
+      <c r="A29" t="s" s="2">
         <v>315</v>
       </c>
-      <c r="B29" t="s" s="15">
+      <c r="B29" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C29" t="s" s="15">
+      <c r="C29" t="s" s="2">
         <v>316</v>
       </c>
-      <c r="D29" t="s" s="15">
+      <c r="D29" t="s" s="2">
         <v>317</v>
       </c>
-      <c r="E29" t="s" s="15">
+      <c r="E29" t="s" s="2">
         <v>318</v>
       </c>
-      <c r="F29" t="s" s="15">
+      <c r="F29" t="s" s="2">
         <v>319</v>
       </c>
-      <c r="G29" t="s" s="15">
+      <c r="G29" t="s" s="2">
         <v>320</v>
       </c>
-      <c r="H29" t="s" s="15">
+      <c r="H29" t="s" s="2">
         <v>321</v>
       </c>
-      <c r="I29" t="s" s="15">
+      <c r="I29" t="s" s="2">
         <v>322</v>
       </c>
-      <c r="J29" t="s" s="15">
+      <c r="J29" t="s" s="2">
         <v>323</v>
       </c>
-      <c r="K29" t="s" s="15">
+      <c r="K29" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L29" t="s" s="15">
+      <c r="L29" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M29" t="s" s="15">
+      <c r="M29" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N29" t="s" s="15">
+      <c r="N29" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O29" t="s" s="15">
+      <c r="O29" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="P29" t="s" s="15">
+      <c r="P29" t="s" s="2">
         <v>228</v>
       </c>
-      <c r="Q29" t="s" s="15">
+      <c r="Q29" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R29" t="s" s="15">
+      <c r="R29" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S29" t="s" s="15">
+      <c r="S29" t="s" s="2">
         <v>324</v>
       </c>
-      <c r="T29" s="11"/>
+      <c r="T29" s="3"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" t="s" s="15">
+      <c r="A30" t="s" s="2">
         <v>325</v>
       </c>
-      <c r="B30" t="s" s="15">
+      <c r="B30" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C30" t="s" s="15">
+      <c r="C30" t="s" s="2">
         <v>326</v>
       </c>
-      <c r="D30" t="s" s="15">
+      <c r="D30" t="s" s="2">
         <v>327</v>
       </c>
-      <c r="E30" t="s" s="15">
+      <c r="E30" t="s" s="2">
         <v>318</v>
       </c>
-      <c r="F30" t="s" s="15">
+      <c r="F30" t="s" s="2">
         <v>328</v>
       </c>
-      <c r="G30" t="s" s="15">
+      <c r="G30" t="s" s="2">
         <v>320</v>
       </c>
-      <c r="H30" t="s" s="15">
+      <c r="H30" t="s" s="2">
         <v>329</v>
       </c>
-      <c r="I30" t="s" s="15">
+      <c r="I30" t="s" s="2">
         <v>330</v>
       </c>
-      <c r="J30" t="s" s="15">
+      <c r="J30" t="s" s="2">
         <v>331</v>
       </c>
-      <c r="K30" t="s" s="15">
+      <c r="K30" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L30" t="s" s="15">
+      <c r="L30" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M30" t="s" s="15">
+      <c r="M30" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N30" t="s" s="15">
+      <c r="N30" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O30" t="s" s="15">
+      <c r="O30" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="P30" t="s" s="15">
+      <c r="P30" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="Q30" t="s" s="15">
+      <c r="Q30" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R30" t="s" s="15">
+      <c r="R30" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S30" t="s" s="15">
+      <c r="S30" t="s" s="2">
         <v>332</v>
       </c>
-      <c r="T30" s="11"/>
+      <c r="T30" s="3"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" t="s" s="15">
+      <c r="A31" t="s" s="2">
         <v>333</v>
       </c>
-      <c r="B31" t="s" s="15">
+      <c r="B31" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C31" t="s" s="15">
+      <c r="C31" t="s" s="2">
         <v>334</v>
       </c>
-      <c r="D31" t="s" s="15">
+      <c r="D31" t="s" s="2">
         <v>334</v>
       </c>
-      <c r="E31" t="s" s="15">
+      <c r="E31" t="s" s="2">
         <v>335</v>
       </c>
-      <c r="F31" t="s" s="15">
+      <c r="F31" t="s" s="2">
         <v>336</v>
       </c>
-      <c r="G31" t="s" s="15">
+      <c r="G31" t="s" s="2">
         <v>337</v>
       </c>
-      <c r="H31" t="s" s="15">
+      <c r="H31" t="s" s="2">
         <v>338</v>
       </c>
-      <c r="I31" t="s" s="15">
+      <c r="I31" t="s" s="2">
         <v>339</v>
       </c>
-      <c r="J31" t="s" s="15">
+      <c r="J31" t="s" s="2">
         <v>340</v>
       </c>
-      <c r="K31" t="s" s="15">
+      <c r="K31" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L31" t="s" s="15">
+      <c r="L31" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M31" t="s" s="15">
+      <c r="M31" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N31" t="s" s="15">
+      <c r="N31" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O31" t="s" s="15">
+      <c r="O31" t="s" s="2">
         <v>341</v>
       </c>
-      <c r="P31" t="s" s="15">
+      <c r="P31" t="s" s="2">
         <v>342</v>
       </c>
-      <c r="Q31" t="s" s="15">
+      <c r="Q31" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R31" t="s" s="15">
+      <c r="R31" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S31" s="16"/>
-      <c r="T31" s="11"/>
+      <c r="S31" s="3"/>
+      <c r="T31" s="3"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" t="s" s="15">
+      <c r="A32" t="s" s="2">
         <v>343</v>
       </c>
-      <c r="B32" t="s" s="15">
+      <c r="B32" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C32" t="s" s="15">
+      <c r="C32" t="s" s="2">
         <v>344</v>
       </c>
-      <c r="D32" t="s" s="15">
+      <c r="D32" t="s" s="2">
         <v>344</v>
       </c>
-      <c r="E32" t="s" s="15">
+      <c r="E32" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="F32" t="s" s="15">
+      <c r="F32" t="s" s="2">
         <v>346</v>
       </c>
-      <c r="G32" t="s" s="15">
+      <c r="G32" t="s" s="2">
         <v>347</v>
       </c>
-      <c r="H32" t="s" s="15">
+      <c r="H32" t="s" s="2">
         <v>348</v>
       </c>
-      <c r="I32" t="s" s="15">
+      <c r="I32" t="s" s="2">
         <v>349</v>
       </c>
-      <c r="J32" t="s" s="15">
+      <c r="J32" t="s" s="2">
         <v>350</v>
       </c>
-      <c r="K32" t="s" s="15">
+      <c r="K32" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L32" t="s" s="15">
+      <c r="L32" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M32" t="s" s="15">
+      <c r="M32" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N32" t="s" s="15">
+      <c r="N32" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O32" t="s" s="15">
+      <c r="O32" t="s" s="2">
         <v>314</v>
       </c>
-      <c r="P32" t="s" s="15">
+      <c r="P32" t="s" s="2">
         <v>351</v>
       </c>
-      <c r="Q32" t="s" s="15">
+      <c r="Q32" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R32" t="s" s="15">
+      <c r="R32" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S32" s="16"/>
-      <c r="T32" s="11"/>
+      <c r="S32" s="3"/>
+      <c r="T32" s="3"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" t="s" s="15">
+      <c r="A33" t="s" s="2">
         <v>352</v>
       </c>
-      <c r="B33" t="s" s="15">
+      <c r="B33" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C33" t="s" s="15">
+      <c r="C33" t="s" s="2">
         <v>353</v>
       </c>
-      <c r="D33" t="s" s="15">
+      <c r="D33" t="s" s="2">
         <v>353</v>
       </c>
-      <c r="E33" t="s" s="15">
+      <c r="E33" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="F33" t="s" s="15">
+      <c r="F33" t="s" s="2">
         <v>354</v>
       </c>
-      <c r="G33" t="s" s="15">
+      <c r="G33" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="H33" t="s" s="15">
+      <c r="H33" t="s" s="2">
         <v>355</v>
       </c>
-      <c r="I33" t="s" s="15">
+      <c r="I33" t="s" s="2">
         <v>356</v>
       </c>
-      <c r="J33" t="s" s="15">
+      <c r="J33" t="s" s="2">
         <v>357</v>
       </c>
-      <c r="K33" t="s" s="15">
+      <c r="K33" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L33" t="s" s="15">
+      <c r="L33" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M33" t="s" s="15">
+      <c r="M33" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N33" t="s" s="15">
+      <c r="N33" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O33" t="s" s="15">
+      <c r="O33" t="s" s="2">
         <v>358</v>
       </c>
-      <c r="P33" t="s" s="15">
+      <c r="P33" t="s" s="2">
         <v>359</v>
       </c>
-      <c r="Q33" t="s" s="15">
+      <c r="Q33" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R33" t="s" s="15">
+      <c r="R33" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S33" s="16"/>
-      <c r="T33" s="11"/>
+      <c r="S33" s="3"/>
+      <c r="T33" s="3"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" t="s" s="15">
+      <c r="A34" t="s" s="2">
         <v>360</v>
       </c>
-      <c r="B34" t="s" s="15">
+      <c r="B34" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C34" t="s" s="15">
+      <c r="C34" t="s" s="2">
         <v>361</v>
       </c>
-      <c r="D34" t="s" s="15">
+      <c r="D34" t="s" s="2">
         <v>361</v>
       </c>
-      <c r="E34" t="s" s="15">
+      <c r="E34" t="s" s="2">
         <v>335</v>
       </c>
-      <c r="F34" t="s" s="15">
+      <c r="F34" t="s" s="2">
         <v>362</v>
       </c>
-      <c r="G34" t="s" s="15">
+      <c r="G34" t="s" s="2">
         <v>337</v>
       </c>
-      <c r="H34" t="s" s="15">
+      <c r="H34" t="s" s="2">
         <v>363</v>
       </c>
-      <c r="I34" t="s" s="15">
+      <c r="I34" t="s" s="2">
         <v>364</v>
       </c>
-      <c r="J34" t="s" s="15">
+      <c r="J34" t="s" s="2">
         <v>365</v>
       </c>
-      <c r="K34" t="s" s="15">
+      <c r="K34" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L34" t="s" s="15">
+      <c r="L34" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M34" t="s" s="15">
+      <c r="M34" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N34" t="s" s="15">
+      <c r="N34" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O34" t="s" s="15">
+      <c r="O34" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="P34" t="s" s="15">
+      <c r="P34" t="s" s="2">
         <v>367</v>
       </c>
-      <c r="Q34" t="s" s="15">
+      <c r="Q34" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R34" t="s" s="15">
+      <c r="R34" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S34" s="16"/>
-      <c r="T34" s="11"/>
+      <c r="S34" s="3"/>
+      <c r="T34" s="3"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="A35" t="s" s="15">
+      <c r="A35" t="s" s="2">
         <v>368</v>
       </c>
-      <c r="B35" t="s" s="15">
+      <c r="B35" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C35" t="s" s="15">
+      <c r="C35" t="s" s="2">
         <v>369</v>
       </c>
-      <c r="D35" t="s" s="15">
+      <c r="D35" t="s" s="2">
         <v>369</v>
       </c>
-      <c r="E35" t="s" s="15">
+      <c r="E35" t="s" s="2">
         <v>370</v>
       </c>
-      <c r="F35" t="s" s="15">
+      <c r="F35" t="s" s="2">
         <v>371</v>
       </c>
-      <c r="G35" t="s" s="15">
+      <c r="G35" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="H35" t="s" s="15">
+      <c r="H35" t="s" s="2">
         <v>373</v>
       </c>
-      <c r="I35" t="s" s="15">
+      <c r="I35" t="s" s="2">
         <v>374</v>
       </c>
-      <c r="J35" t="s" s="15">
+      <c r="J35" t="s" s="2">
         <v>375</v>
       </c>
-      <c r="K35" t="s" s="15">
+      <c r="K35" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L35" t="s" s="15">
+      <c r="L35" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M35" t="s" s="15">
+      <c r="M35" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N35" t="s" s="15">
+      <c r="N35" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O35" t="s" s="15">
+      <c r="O35" t="s" s="2">
         <v>218</v>
       </c>
-      <c r="P35" t="s" s="15">
+      <c r="P35" t="s" s="2">
         <v>376</v>
       </c>
-      <c r="Q35" t="s" s="15">
+      <c r="Q35" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R35" t="s" s="15">
+      <c r="R35" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S35" s="16"/>
-      <c r="T35" s="11"/>
+      <c r="S35" s="3"/>
+      <c r="T35" s="3"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="A36" t="s" s="15">
+      <c r="A36" t="s" s="2">
         <v>377</v>
       </c>
-      <c r="B36" t="s" s="15">
+      <c r="B36" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C36" t="s" s="15">
+      <c r="C36" t="s" s="2">
         <v>378</v>
       </c>
-      <c r="D36" t="s" s="15">
+      <c r="D36" t="s" s="2">
         <v>378</v>
       </c>
-      <c r="E36" t="s" s="15">
+      <c r="E36" t="s" s="2">
         <v>279</v>
       </c>
-      <c r="F36" t="s" s="15">
+      <c r="F36" t="s" s="2">
         <v>379</v>
       </c>
-      <c r="G36" t="s" s="15">
+      <c r="G36" t="s" s="2">
         <v>281</v>
       </c>
-      <c r="H36" t="s" s="15">
+      <c r="H36" t="s" s="2">
         <v>380</v>
       </c>
-      <c r="I36" t="s" s="15">
+      <c r="I36" t="s" s="2">
         <v>381</v>
       </c>
-      <c r="J36" t="s" s="15">
+      <c r="J36" t="s" s="2">
         <v>382</v>
       </c>
-      <c r="K36" t="s" s="15">
+      <c r="K36" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L36" t="s" s="15">
+      <c r="L36" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M36" t="s" s="15">
+      <c r="M36" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N36" t="s" s="15">
+      <c r="N36" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O36" t="s" s="15">
+      <c r="O36" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="P36" s="17">
+      <c r="P36" s="5">
         <v>18.3333333333333</v>
       </c>
-      <c r="Q36" t="s" s="15">
+      <c r="Q36" t="s" s="2">
         <v>384</v>
       </c>
-      <c r="R36" t="s" s="15">
+      <c r="R36" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S36" t="s" s="15">
+      <c r="S36" t="s" s="2">
         <v>385</v>
       </c>
-      <c r="T36" s="11"/>
+      <c r="T36" s="3"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="A37" t="s" s="15">
+      <c r="A37" t="s" s="2">
         <v>386</v>
       </c>
-      <c r="B37" t="s" s="15">
+      <c r="B37" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C37" t="s" s="15">
+      <c r="C37" t="s" s="2">
         <v>387</v>
       </c>
-      <c r="D37" t="s" s="15">
+      <c r="D37" t="s" s="2">
         <v>387</v>
       </c>
-      <c r="E37" t="s" s="15">
+      <c r="E37" t="s" s="2">
         <v>388</v>
       </c>
-      <c r="F37" t="s" s="15">
+      <c r="F37" t="s" s="2">
         <v>389</v>
       </c>
-      <c r="G37" t="s" s="15">
+      <c r="G37" t="s" s="2">
         <v>390</v>
       </c>
-      <c r="H37" t="s" s="15">
+      <c r="H37" t="s" s="2">
         <v>391</v>
       </c>
-      <c r="I37" t="s" s="15">
+      <c r="I37" t="s" s="2">
         <v>392</v>
       </c>
-      <c r="J37" t="s" s="15">
+      <c r="J37" t="s" s="2">
         <v>393</v>
       </c>
-      <c r="K37" t="s" s="15">
+      <c r="K37" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L37" t="s" s="15">
+      <c r="L37" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M37" t="s" s="15">
+      <c r="M37" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N37" t="s" s="15">
+      <c r="N37" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O37" t="s" s="15">
+      <c r="O37" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="P37" t="s" s="15">
+      <c r="P37" t="s" s="2">
         <v>394</v>
       </c>
-      <c r="Q37" t="s" s="15">
+      <c r="Q37" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R37" t="s" s="15">
+      <c r="R37" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S37" s="16"/>
-      <c r="T37" s="11"/>
+      <c r="S37" s="3"/>
+      <c r="T37" s="3"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="A38" t="s" s="15">
+      <c r="A38" t="s" s="2">
         <v>395</v>
       </c>
-      <c r="B38" t="s" s="15">
+      <c r="B38" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" t="s" s="15">
+      <c r="C38" s="3"/>
+      <c r="D38" t="s" s="2">
         <v>396</v>
       </c>
-      <c r="E38" t="s" s="15">
+      <c r="E38" t="s" s="2">
         <v>397</v>
       </c>
-      <c r="F38" t="s" s="15">
+      <c r="F38" t="s" s="2">
         <v>398</v>
       </c>
-      <c r="G38" t="s" s="15">
+      <c r="G38" t="s" s="2">
         <v>399</v>
       </c>
-      <c r="H38" t="s" s="15">
+      <c r="H38" t="s" s="2">
         <v>400</v>
       </c>
-      <c r="I38" t="s" s="15">
+      <c r="I38" t="s" s="2">
         <v>401</v>
       </c>
-      <c r="J38" t="s" s="15">
+      <c r="J38" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="K38" t="s" s="15">
+      <c r="K38" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L38" t="s" s="15">
+      <c r="L38" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M38" t="s" s="15">
+      <c r="M38" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N38" t="s" s="15">
+      <c r="N38" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O38" t="s" s="15">
+      <c r="O38" t="s" s="2">
         <v>403</v>
       </c>
-      <c r="P38" t="s" s="15">
+      <c r="P38" t="s" s="2">
         <v>404</v>
       </c>
-      <c r="Q38" t="s" s="15">
+      <c r="Q38" t="s" s="2">
         <v>256</v>
       </c>
-      <c r="R38" t="s" s="15">
+      <c r="R38" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S38" t="s" s="15">
+      <c r="S38" t="s" s="2">
         <v>405</v>
       </c>
-      <c r="T38" s="11"/>
+      <c r="T38" s="3"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" t="s" s="15">
+      <c r="A39" t="s" s="2">
         <v>406</v>
       </c>
-      <c r="B39" t="s" s="15">
+      <c r="B39" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C39" t="s" s="15">
+      <c r="C39" t="s" s="2">
         <v>407</v>
       </c>
-      <c r="D39" t="s" s="15">
+      <c r="D39" t="s" s="2">
         <v>407</v>
       </c>
-      <c r="E39" t="s" s="15">
+      <c r="E39" t="s" s="2">
         <v>408</v>
       </c>
-      <c r="F39" t="s" s="15">
+      <c r="F39" t="s" s="2">
         <v>409</v>
       </c>
-      <c r="G39" t="s" s="15">
+      <c r="G39" t="s" s="2">
         <v>410</v>
       </c>
-      <c r="H39" t="s" s="15">
+      <c r="H39" t="s" s="2">
         <v>411</v>
       </c>
-      <c r="I39" t="s" s="15">
+      <c r="I39" t="s" s="2">
         <v>412</v>
       </c>
-      <c r="J39" t="s" s="15">
+      <c r="J39" t="s" s="2">
         <v>413</v>
       </c>
-      <c r="K39" t="s" s="15">
+      <c r="K39" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L39" t="s" s="15">
+      <c r="L39" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M39" t="s" s="15">
+      <c r="M39" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N39" t="s" s="15">
+      <c r="N39" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O39" t="s" s="15">
+      <c r="O39" t="s" s="2">
         <v>414</v>
       </c>
-      <c r="P39" t="s" s="15">
+      <c r="P39" t="s" s="2">
         <v>394</v>
       </c>
-      <c r="Q39" t="s" s="15">
+      <c r="Q39" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R39" t="s" s="15">
+      <c r="R39" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S39" s="16"/>
-      <c r="T39" s="11"/>
+      <c r="S39" s="3"/>
+      <c r="T39" s="3"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" t="s" s="15">
+      <c r="A40" t="s" s="2">
         <v>415</v>
       </c>
-      <c r="B40" t="s" s="15">
+      <c r="B40" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C40" t="s" s="15">
+      <c r="C40" t="s" s="2">
         <v>416</v>
       </c>
-      <c r="D40" t="s" s="15">
+      <c r="D40" t="s" s="2">
         <v>416</v>
       </c>
-      <c r="E40" t="s" s="15">
+      <c r="E40" t="s" s="2">
         <v>417</v>
       </c>
-      <c r="F40" t="s" s="15">
+      <c r="F40" t="s" s="2">
         <v>418</v>
       </c>
-      <c r="G40" t="s" s="15">
+      <c r="G40" t="s" s="2">
         <v>419</v>
       </c>
-      <c r="H40" t="s" s="15">
+      <c r="H40" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="I40" t="s" s="15">
+      <c r="I40" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="J40" t="s" s="15">
+      <c r="J40" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="K40" t="s" s="15">
+      <c r="K40" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L40" t="s" s="15">
+      <c r="L40" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M40" t="s" s="15">
+      <c r="M40" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N40" t="s" s="15">
+      <c r="N40" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O40" t="s" s="15">
+      <c r="O40" t="s" s="2">
         <v>296</v>
       </c>
-      <c r="P40" t="s" s="15">
+      <c r="P40" t="s" s="2">
         <v>423</v>
       </c>
-      <c r="Q40" t="s" s="15">
+      <c r="Q40" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R40" t="s" s="15">
+      <c r="R40" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S40" s="16"/>
-      <c r="T40" s="11"/>
+      <c r="S40" s="3"/>
+      <c r="T40" s="3"/>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" t="s" s="15">
+      <c r="A41" t="s" s="2">
         <v>424</v>
       </c>
-      <c r="B41" t="s" s="15">
+      <c r="B41" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C41" t="s" s="15">
+      <c r="C41" t="s" s="2">
         <v>425</v>
       </c>
-      <c r="D41" t="s" s="15">
+      <c r="D41" t="s" s="2">
         <v>425</v>
       </c>
-      <c r="E41" t="s" s="15">
+      <c r="E41" t="s" s="2">
         <v>426</v>
       </c>
-      <c r="F41" t="s" s="15">
+      <c r="F41" t="s" s="2">
         <v>427</v>
       </c>
-      <c r="G41" t="s" s="15">
+      <c r="G41" t="s" s="2">
         <v>428</v>
       </c>
-      <c r="H41" t="s" s="15">
+      <c r="H41" t="s" s="2">
         <v>429</v>
       </c>
-      <c r="I41" t="s" s="15">
+      <c r="I41" t="s" s="2">
         <v>430</v>
       </c>
-      <c r="J41" t="s" s="15">
+      <c r="J41" t="s" s="2">
         <v>431</v>
       </c>
-      <c r="K41" t="s" s="15">
+      <c r="K41" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L41" t="s" s="15">
+      <c r="L41" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M41" t="s" s="15">
+      <c r="M41" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N41" t="s" s="15">
+      <c r="N41" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O41" t="s" s="15">
+      <c r="O41" t="s" s="2">
         <v>432</v>
       </c>
-      <c r="P41" t="s" s="15">
+      <c r="P41" t="s" s="2">
         <v>433</v>
       </c>
-      <c r="Q41" t="s" s="15">
+      <c r="Q41" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R41" t="s" s="15">
+      <c r="R41" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S41" s="16"/>
-      <c r="T41" s="11"/>
+      <c r="S41" s="3"/>
+      <c r="T41" s="3"/>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" t="s" s="15">
+      <c r="A42" t="s" s="2">
         <v>434</v>
       </c>
-      <c r="B42" t="s" s="15">
+      <c r="B42" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C42" t="s" s="15">
+      <c r="C42" t="s" s="2">
         <v>435</v>
       </c>
-      <c r="D42" t="s" s="15">
+      <c r="D42" t="s" s="2">
         <v>435</v>
       </c>
-      <c r="E42" t="s" s="15">
+      <c r="E42" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="F42" t="s" s="15">
+      <c r="F42" t="s" s="2">
         <v>436</v>
       </c>
-      <c r="G42" t="s" s="15">
+      <c r="G42" t="s" s="2">
         <v>437</v>
       </c>
-      <c r="H42" t="s" s="15">
+      <c r="H42" t="s" s="2">
         <v>438</v>
       </c>
-      <c r="I42" t="s" s="15">
+      <c r="I42" t="s" s="2">
         <v>439</v>
       </c>
-      <c r="J42" t="s" s="15">
+      <c r="J42" t="s" s="2">
         <v>440</v>
       </c>
-      <c r="K42" t="s" s="15">
+      <c r="K42" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L42" t="s" s="15">
+      <c r="L42" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M42" t="s" s="15">
+      <c r="M42" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N42" t="s" s="15">
+      <c r="N42" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O42" t="s" s="15">
+      <c r="O42" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="P42" t="s" s="15">
+      <c r="P42" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="Q42" t="s" s="15">
+      <c r="Q42" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R42" t="s" s="15">
+      <c r="R42" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S42" s="16"/>
-      <c r="T42" s="11"/>
+      <c r="S42" s="3"/>
+      <c r="T42" s="3"/>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" t="s" s="15">
+      <c r="A43" t="s" s="2">
         <v>441</v>
       </c>
-      <c r="B43" t="s" s="15">
+      <c r="B43" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C43" t="s" s="15">
+      <c r="C43" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="D43" t="s" s="15">
+      <c r="D43" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="E43" t="s" s="15">
+      <c r="E43" t="s" s="2">
         <v>290</v>
       </c>
-      <c r="F43" t="s" s="15">
+      <c r="F43" t="s" s="2">
         <v>443</v>
       </c>
-      <c r="G43" t="s" s="15">
+      <c r="G43" t="s" s="2">
         <v>444</v>
       </c>
-      <c r="H43" t="s" s="15">
+      <c r="H43" t="s" s="2">
         <v>445</v>
       </c>
-      <c r="I43" t="s" s="15">
+      <c r="I43" t="s" s="2">
         <v>446</v>
       </c>
-      <c r="J43" t="s" s="15">
+      <c r="J43" t="s" s="2">
         <v>447</v>
       </c>
-      <c r="K43" t="s" s="15">
+      <c r="K43" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L43" t="s" s="15">
+      <c r="L43" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M43" t="s" s="15">
+      <c r="M43" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N43" t="s" s="15">
+      <c r="N43" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O43" t="s" s="15">
+      <c r="O43" t="s" s="2">
         <v>448</v>
       </c>
-      <c r="P43" t="s" s="15">
+      <c r="P43" t="s" s="2">
         <v>449</v>
       </c>
-      <c r="Q43" t="s" s="15">
+      <c r="Q43" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R43" t="s" s="15">
+      <c r="R43" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S43" s="16"/>
-      <c r="T43" s="11"/>
+      <c r="S43" s="3"/>
+      <c r="T43" s="3"/>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="A44" t="s" s="15">
+      <c r="A44" t="s" s="2">
         <v>450</v>
       </c>
-      <c r="B44" t="s" s="15">
+      <c r="B44" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C44" t="s" s="15">
+      <c r="C44" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="D44" t="s" s="15">
+      <c r="D44" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="E44" t="s" s="15">
+      <c r="E44" t="s" s="2">
         <v>452</v>
       </c>
-      <c r="F44" t="s" s="15">
+      <c r="F44" t="s" s="2">
         <v>453</v>
       </c>
-      <c r="G44" t="s" s="15">
+      <c r="G44" t="s" s="2">
         <v>454</v>
       </c>
-      <c r="H44" t="s" s="15">
+      <c r="H44" t="s" s="2">
         <v>455</v>
       </c>
-      <c r="I44" t="s" s="15">
+      <c r="I44" t="s" s="2">
         <v>456</v>
       </c>
-      <c r="J44" t="s" s="15">
+      <c r="J44" t="s" s="2">
         <v>457</v>
       </c>
-      <c r="K44" t="s" s="15">
+      <c r="K44" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L44" t="s" s="15">
+      <c r="L44" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M44" t="s" s="15">
+      <c r="M44" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N44" t="s" s="15">
+      <c r="N44" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O44" t="s" s="15">
+      <c r="O44" t="s" s="2">
         <v>314</v>
       </c>
-      <c r="P44" t="s" s="15">
+      <c r="P44" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="Q44" t="s" s="15">
+      <c r="Q44" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R44" t="s" s="15">
+      <c r="R44" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S44" s="16"/>
-      <c r="T44" s="11"/>
+      <c r="S44" s="3"/>
+      <c r="T44" s="3"/>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="A45" t="s" s="15">
+      <c r="A45" t="s" s="2">
         <v>459</v>
       </c>
-      <c r="B45" t="s" s="15">
+      <c r="B45" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C45" t="s" s="15">
+      <c r="C45" t="s" s="2">
         <v>460</v>
       </c>
-      <c r="D45" t="s" s="15">
+      <c r="D45" t="s" s="2">
         <v>460</v>
       </c>
-      <c r="E45" t="s" s="15">
+      <c r="E45" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="F45" t="s" s="15">
+      <c r="F45" t="s" s="2">
         <v>461</v>
       </c>
-      <c r="G45" t="s" s="15">
+      <c r="G45" t="s" s="2">
         <v>347</v>
       </c>
-      <c r="H45" t="s" s="15">
+      <c r="H45" t="s" s="2">
         <v>462</v>
       </c>
-      <c r="I45" t="s" s="15">
+      <c r="I45" t="s" s="2">
         <v>463</v>
       </c>
-      <c r="J45" t="s" s="15">
+      <c r="J45" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="K45" t="s" s="15">
+      <c r="K45" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L45" t="s" s="15">
+      <c r="L45" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M45" t="s" s="15">
+      <c r="M45" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N45" t="s" s="15">
+      <c r="N45" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O45" t="s" s="15">
+      <c r="O45" t="s" s="2">
         <v>414</v>
       </c>
-      <c r="P45" t="s" s="15">
+      <c r="P45" t="s" s="2">
         <v>297</v>
       </c>
-      <c r="Q45" t="s" s="15">
+      <c r="Q45" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R45" t="s" s="15">
+      <c r="R45" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S45" s="16"/>
-      <c r="T45" s="11"/>
+      <c r="S45" s="3"/>
+      <c r="T45" s="3"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="A46" t="s" s="15">
+      <c r="A46" t="s" s="2">
         <v>465</v>
       </c>
-      <c r="B46" t="s" s="15">
+      <c r="B46" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C46" t="s" s="15">
+      <c r="C46" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="D46" t="s" s="15">
+      <c r="D46" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="E46" t="s" s="15">
+      <c r="E46" t="s" s="2">
         <v>467</v>
       </c>
-      <c r="F46" t="s" s="15">
+      <c r="F46" t="s" s="2">
         <v>468</v>
       </c>
-      <c r="G46" t="s" s="15">
+      <c r="G46" t="s" s="2">
         <v>469</v>
       </c>
-      <c r="H46" t="s" s="15">
+      <c r="H46" t="s" s="2">
         <v>470</v>
       </c>
-      <c r="I46" t="s" s="15">
+      <c r="I46" t="s" s="2">
         <v>471</v>
       </c>
-      <c r="J46" t="s" s="15">
+      <c r="J46" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="K46" t="s" s="15">
+      <c r="K46" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L46" t="s" s="15">
+      <c r="L46" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M46" t="s" s="15">
+      <c r="M46" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N46" t="s" s="15">
+      <c r="N46" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O46" t="s" s="15">
+      <c r="O46" t="s" s="2">
         <v>313</v>
       </c>
-      <c r="P46" t="s" s="15">
+      <c r="P46" t="s" s="2">
         <v>473</v>
       </c>
-      <c r="Q46" t="s" s="15">
+      <c r="Q46" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R46" t="s" s="15">
+      <c r="R46" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S46" s="16"/>
-      <c r="T46" s="11"/>
+      <c r="S46" s="3"/>
+      <c r="T46" s="3"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="A47" t="s" s="15">
+      <c r="A47" t="s" s="2">
         <v>474</v>
       </c>
-      <c r="B47" t="s" s="15">
+      <c r="B47" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C47" t="s" s="15">
+      <c r="C47" t="s" s="2">
         <v>475</v>
       </c>
-      <c r="D47" t="s" s="15">
+      <c r="D47" t="s" s="2">
         <v>475</v>
       </c>
-      <c r="E47" t="s" s="15">
+      <c r="E47" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="F47" t="s" s="15">
+      <c r="F47" t="s" s="2">
         <v>476</v>
       </c>
-      <c r="G47" t="s" s="15">
+      <c r="G47" t="s" s="2">
         <v>437</v>
       </c>
-      <c r="H47" t="s" s="15">
+      <c r="H47" t="s" s="2">
         <v>477</v>
       </c>
-      <c r="I47" t="s" s="15">
+      <c r="I47" t="s" s="2">
         <v>478</v>
       </c>
-      <c r="J47" t="s" s="15">
+      <c r="J47" t="s" s="2">
         <v>479</v>
       </c>
-      <c r="K47" t="s" s="15">
+      <c r="K47" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L47" t="s" s="15">
+      <c r="L47" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M47" t="s" s="15">
+      <c r="M47" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N47" t="s" s="15">
+      <c r="N47" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O47" t="s" s="15">
+      <c r="O47" t="s" s="2">
         <v>313</v>
       </c>
-      <c r="P47" t="s" s="15">
+      <c r="P47" t="s" s="2">
         <v>414</v>
       </c>
-      <c r="Q47" t="s" s="15">
+      <c r="Q47" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R47" t="s" s="15">
+      <c r="R47" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S47" s="16"/>
-      <c r="T47" s="11"/>
+      <c r="S47" s="3"/>
+      <c r="T47" s="3"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" t="s" s="15">
+      <c r="A48" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="B48" t="s" s="15">
+      <c r="B48" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C48" t="s" s="15">
+      <c r="C48" t="s" s="2">
         <v>481</v>
       </c>
-      <c r="D48" t="s" s="15">
+      <c r="D48" t="s" s="2">
         <v>481</v>
       </c>
-      <c r="E48" t="s" s="15">
+      <c r="E48" t="s" s="2">
         <v>250</v>
       </c>
-      <c r="F48" t="s" s="15">
+      <c r="F48" t="s" s="2">
         <v>482</v>
       </c>
-      <c r="G48" t="s" s="15">
+      <c r="G48" t="s" s="2">
         <v>483</v>
       </c>
-      <c r="H48" t="s" s="15">
+      <c r="H48" t="s" s="2">
         <v>484</v>
       </c>
-      <c r="I48" t="s" s="15">
+      <c r="I48" t="s" s="2">
         <v>485</v>
       </c>
-      <c r="J48" t="s" s="15">
+      <c r="J48" t="s" s="2">
         <v>486</v>
       </c>
-      <c r="K48" t="s" s="15">
+      <c r="K48" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L48" t="s" s="15">
+      <c r="L48" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M48" t="s" s="15">
+      <c r="M48" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N48" t="s" s="15">
+      <c r="N48" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O48" t="s" s="15">
+      <c r="O48" t="s" s="2">
         <v>449</v>
       </c>
-      <c r="P48" t="s" s="15">
+      <c r="P48" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="Q48" t="s" s="15">
+      <c r="Q48" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R48" t="s" s="15">
+      <c r="R48" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S48" s="16"/>
-      <c r="T48" s="11"/>
+      <c r="S48" s="3"/>
+      <c r="T48" s="3"/>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" t="s" s="15">
+      <c r="A49" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="B49" t="s" s="15">
+      <c r="B49" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C49" t="s" s="15">
+      <c r="C49" t="s" s="2">
         <v>488</v>
       </c>
-      <c r="D49" t="s" s="15">
+      <c r="D49" t="s" s="2">
         <v>488</v>
       </c>
-      <c r="E49" t="s" s="15">
+      <c r="E49" t="s" s="2">
         <v>489</v>
       </c>
-      <c r="F49" t="s" s="15">
+      <c r="F49" t="s" s="2">
         <v>490</v>
       </c>
-      <c r="G49" t="s" s="15">
+      <c r="G49" t="s" s="2">
         <v>491</v>
       </c>
-      <c r="H49" t="s" s="15">
+      <c r="H49" t="s" s="2">
         <v>492</v>
       </c>
-      <c r="I49" t="s" s="15">
+      <c r="I49" t="s" s="2">
         <v>493</v>
       </c>
-      <c r="J49" t="s" s="15">
+      <c r="J49" t="s" s="2">
         <v>494</v>
       </c>
-      <c r="K49" t="s" s="15">
+      <c r="K49" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L49" t="s" s="15">
+      <c r="L49" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M49" t="s" s="15">
+      <c r="M49" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="N49" t="s" s="15">
+      <c r="N49" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O49" t="s" s="15">
+      <c r="O49" t="s" s="2">
         <v>495</v>
       </c>
-      <c r="P49" t="s" s="15">
+      <c r="P49" t="s" s="2">
         <v>496</v>
       </c>
-      <c r="Q49" t="s" s="15">
+      <c r="Q49" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R49" t="s" s="15">
+      <c r="R49" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S49" s="16"/>
-      <c r="T49" s="11"/>
+      <c r="S49" s="3"/>
+      <c r="T49" s="3"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="A50" t="s" s="15">
+      <c r="A50" t="s" s="2">
         <v>497</v>
       </c>
-      <c r="B50" t="s" s="15">
+      <c r="B50" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="C50" t="s" s="15">
+      <c r="C50" t="s" s="2">
         <v>498</v>
       </c>
-      <c r="D50" t="s" s="15">
+      <c r="D50" t="s" s="2">
         <v>498</v>
       </c>
-      <c r="E50" t="s" s="15">
+      <c r="E50" t="s" s="2">
         <v>499</v>
       </c>
-      <c r="F50" t="s" s="15">
+      <c r="F50" t="s" s="2">
         <v>500</v>
       </c>
-      <c r="G50" t="s" s="15">
+      <c r="G50" t="s" s="2">
         <v>501</v>
       </c>
-      <c r="H50" t="s" s="15">
+      <c r="H50" t="s" s="2">
         <v>502</v>
       </c>
-      <c r="I50" t="s" s="15">
+      <c r="I50" t="s" s="2">
         <v>503</v>
       </c>
-      <c r="J50" t="s" s="15">
+      <c r="J50" t="s" s="2">
         <v>504</v>
       </c>
-      <c r="K50" t="s" s="15">
+      <c r="K50" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="L50" t="s" s="15">
+      <c r="L50" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="M50" t="s" s="15">
+      <c r="M50" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="N50" t="s" s="15">
+      <c r="N50" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="O50" t="s" s="15">
+      <c r="O50" t="s" s="2">
         <v>505</v>
       </c>
-      <c r="P50" t="s" s="15">
+      <c r="P50" t="s" s="2">
         <v>383</v>
       </c>
-      <c r="Q50" t="s" s="15">
+      <c r="Q50" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="R50" t="s" s="15">
+      <c r="R50" t="s" s="2">
         <v>84</v>
       </c>
-      <c r="S50" s="16"/>
-      <c r="T50" s="11"/>
+      <c r="S50" s="3"/>
+      <c r="T50" s="3"/>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="A51" s="18"/>
-      <c r="B51" s="18"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18"/>
-      <c r="F51" s="18"/>
-      <c r="G51" s="18"/>
-      <c r="H51" s="18"/>
-      <c r="I51" s="18"/>
-      <c r="J51" s="18"/>
-      <c r="K51" s="18"/>
-      <c r="L51" s="18"/>
-      <c r="M51" s="18"/>
-      <c r="N51" s="18"/>
-      <c r="O51" s="18"/>
-      <c r="P51" s="18"/>
-      <c r="Q51" s="18"/>
-      <c r="R51" s="18"/>
-      <c r="S51" s="18"/>
-      <c r="T51" s="4"/>
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
+      <c r="O51" s="3"/>
+      <c r="P51" s="3"/>
+      <c r="Q51" s="3"/>
+      <c r="R51" s="3"/>
+      <c r="S51" s="3"/>
+      <c r="T51" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>